<commit_message>
Updated cbc as per 14 days building and 3 months curing pde data
</commit_message>
<xml_diff>
--- a/load_demand.xlsx
+++ b/load_demand.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,729 +436,1561 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1225121715115SSTL0</t>
+          <t>1225119015010QSTL0</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1431</v>
+        <v>1703</v>
       </c>
       <c r="C2" t="n">
-        <v>0.5151997854652722</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1225121716010SXC10</t>
+          <t>1225121715115SSTL0</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>184</v>
+        <v>5668</v>
       </c>
       <c r="C3" t="n">
-        <v>0.5041324751944221</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1225170015010LSTL0</t>
+          <t>1225121716010SXC10</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2471</v>
+        <v>1991</v>
       </c>
       <c r="C4" t="n">
-        <v>0.4306114239742558</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1225170015012LSTL0</t>
+          <t>1225121Z14112LSTL0</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>61107</v>
+        <v>1787</v>
       </c>
       <c r="C5" t="n">
-        <v>0.6340842048806651</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1225221715115SSTL0</t>
+          <t>1225170015010LSTL0</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1375</v>
+        <v>5200</v>
       </c>
       <c r="C6" t="n">
-        <v>0.5205604719764012</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1225221716010SXC10</t>
+          <t>1225170015012LSTL0</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>342</v>
+        <v>65500</v>
       </c>
       <c r="C7" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1225223516121PSKP0</t>
+          <t>1225219015008SLTB0</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10431</v>
+        <v>346</v>
       </c>
       <c r="C8" t="n">
-        <v>0.5080986859747921</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1325114812074TUHL0</t>
+          <t>1225219015010QSTL0</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>19137</v>
+        <v>2900</v>
       </c>
       <c r="C9" t="n">
-        <v>0.553633681952266</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1325119015008SRBT0</t>
+          <t>1225220Z16008RXC10</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>9540</v>
+        <v>242</v>
       </c>
       <c r="C10" t="n">
-        <v>0.5321802091713597</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1325119815106QBRQ0</t>
+          <t>1225221615008QXC10</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>5141</v>
+        <v>615</v>
       </c>
       <c r="C11" t="n">
-        <v>0.5001582193617592</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1325123715105SBRT0</t>
+          <t>1225221715115SSTL0</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4525</v>
+        <v>14167</v>
       </c>
       <c r="C12" t="n">
-        <v>0.5174309466344864</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1325213612065SULX1</t>
+          <t>1225221716010SXC10</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>523</v>
+        <v>1320</v>
       </c>
       <c r="C13" t="n">
-        <v>0.5020166264414052</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1325213615099MSXT0</t>
+          <t>1225222615008RXC10</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>860</v>
+        <v>93</v>
       </c>
       <c r="C14" t="n">
-        <v>0.4394609814963797</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1325214812074TUHL0</t>
+          <t>1225222716121MXC11</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>25972</v>
+        <v>1079</v>
       </c>
       <c r="C15" t="n">
-        <v>0.5724054706355591</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1325214813075STMX0</t>
+          <t>1225222716121NXC11</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2480</v>
+        <v>200</v>
       </c>
       <c r="C16" t="n">
-        <v>0.5077768838830786</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1325214813075SUNE1</t>
+          <t>1225223516121PSKP0</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>64982</v>
+        <v>11420</v>
       </c>
       <c r="C17" t="n">
-        <v>0.6166666666666667</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1325215513073TUHL0</t>
+          <t>1225223516121RBVN0</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>39</v>
+        <v>711</v>
       </c>
       <c r="C18" t="n">
-        <v>0.5207750067042103</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1325215613075TUHL0</t>
+          <t>1325114613071TTMX0</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>8340</v>
+        <v>148</v>
       </c>
       <c r="C19" t="n">
-        <v>0.5246714936980423</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1325215813079STMX0</t>
+          <t>1325114812074TUHL0</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>8563</v>
+        <v>20000</v>
       </c>
       <c r="C20" t="n">
-        <v>0.526816840976133</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1325215813079SUHL0</t>
+          <t>1325119015008SRBT0</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>10540</v>
+        <v>12000</v>
       </c>
       <c r="C21" t="n">
-        <v>0.5321802091713597</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1325216513077TUHL0</t>
+          <t>1325119815106QBRQ0</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1029</v>
+        <v>5889.000000000001</v>
       </c>
       <c r="C22" t="n">
-        <v>0.5080584607133279</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1325216514079TTMX0</t>
+          <t>1325121715100SBRT0</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>5198</v>
+        <v>4000</v>
       </c>
       <c r="C23" t="n">
-        <v>0.5142611960311075</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1325216614081STMX0</t>
+          <t>1325121715100SRBT0</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>5131</v>
+        <v>4569</v>
       </c>
       <c r="C24" t="n">
-        <v>0.5177902923035667</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1325216614081SUTR0</t>
+          <t>1325121715100SRXT0</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>5213</v>
+        <v>3188</v>
       </c>
       <c r="C25" t="n">
-        <v>0.5157307589165996</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1325216814085STMX0</t>
+          <t>1325121715115SLTB0</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>13715</v>
+        <v>4770</v>
       </c>
       <c r="C26" t="n">
-        <v>0.5375435773665862</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1325216814085SURL0</t>
+          <t>1325123715105SBRT0</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>427</v>
+        <v>6500</v>
       </c>
       <c r="C27" t="n">
-        <v>0.5162939125770984</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1325216814085SUTR0</t>
+          <t>1325123715105SRXT0</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>4226</v>
+        <v>900</v>
       </c>
       <c r="C28" t="n">
-        <v>0.5138938053097345</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1325216814085TURL0</t>
+          <t>1325213612065SULX1</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>5113</v>
+        <v>752</v>
       </c>
       <c r="C29" t="n">
-        <v>0.5137114507910968</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1325217413077TUSP0</t>
+          <t>1325213615099MSXT0</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>3844</v>
+        <v>8500</v>
       </c>
       <c r="C30" t="n">
-        <v>0.5152936444086886</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1325217514082HURL2</t>
+          <t>1325214612069TUHL0</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1033</v>
+        <v>6000</v>
       </c>
       <c r="C31" t="n">
-        <v>0.3396674711718959</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1325217514082TTMX0</t>
+          <t>1325214613071TTMX0</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>6492</v>
+        <v>289</v>
       </c>
       <c r="C32" t="n">
-        <v>0.5174094931617056</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1325217613082TUNE0</t>
+          <t>1325214812074TUHL0</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>432</v>
+        <v>27000</v>
       </c>
       <c r="C33" t="n">
-        <v>0.3446017699115044</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1325217613082TUNE2</t>
+          <t>1325214813075STMX0</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2411</v>
+        <v>2900</v>
       </c>
       <c r="C34" t="n">
-        <v>0.3403539823008849</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1325217614084HURL2</t>
+          <t>1325214813075SUNE1</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1036</v>
+        <v>74580</v>
       </c>
       <c r="C35" t="n">
-        <v>0.3368061142397425</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>1325218514086HURL0</t>
+          <t>1325215513073TUHL0</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>2284</v>
+        <v>7747</v>
       </c>
       <c r="C36" t="n">
-        <v>0.5067042102440332</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1325218515088HTMX0</t>
+          <t>1325215613075TTMX0</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>11236</v>
+        <v>4239</v>
       </c>
       <c r="C37" t="n">
-        <v>0.5321802091713597</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>1325218515088TURL0</t>
+          <t>1325215613075TUHL0</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>1717</v>
+        <v>9200</v>
       </c>
       <c r="C38" t="n">
-        <v>0.505728077232502</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>1325219316087VUTR0</t>
+          <t>1325215813079STMX0</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>4822</v>
+        <v>10000</v>
       </c>
       <c r="C39" t="n">
-        <v>0.5187717886832931</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>1325219416089HRHE0</t>
+          <t>1325215813079SUHL0</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>15730</v>
+        <v>12000</v>
       </c>
       <c r="C40" t="n">
-        <v>0.5134084204880665</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>1325219515091VZEP0</t>
+          <t>1325216513077TUHL0</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>112</v>
+        <v>3005</v>
       </c>
       <c r="C41" t="n">
-        <v>0.3358836149101636</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>1325220416092VURL0</t>
+          <t>1325216514079TTMX0</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>840</v>
+        <v>5318</v>
       </c>
       <c r="C42" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>1325220515094VTMX0</t>
+          <t>1325216614081STMX0</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>546</v>
+        <v>6634</v>
       </c>
       <c r="C43" t="n">
-        <v>0.5017457763475462</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>1325220515094VUTR0</t>
+          <t>1325216614081SUTR0</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>5740</v>
+        <v>5866</v>
       </c>
       <c r="C44" t="n">
-        <v>0.5163529096272459</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>1325220516095HTMX0</t>
+          <t>1325216614081TVECE</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>3866</v>
+        <v>290</v>
       </c>
       <c r="C45" t="n">
-        <v>0.5134084204880665</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>1325220516095HUTR0</t>
+          <t>1325216813083TUNE0</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>636</v>
+        <v>4000</v>
       </c>
       <c r="C46" t="n">
-        <v>0.5042531509788147</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>1325221416095VURL0</t>
+          <t>1325216814085STMX0</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>11151</v>
+        <v>14000</v>
       </c>
       <c r="C47" t="n">
-        <v>0.5321802091713597</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>1325221417100HURL1</t>
+          <t>1325216814085SURL0</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>16836</v>
+        <v>6076</v>
       </c>
       <c r="C48" t="n">
-        <v>0.5455886296594261</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>1325221715100SRHT0</t>
+          <t>1325216814085SUTR0</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>18097</v>
+        <v>5181</v>
       </c>
       <c r="C49" t="n">
-        <v>0.5509519978546528</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>1325223517104HRHT0</t>
+          <t>1325216814085TURL0</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>7726</v>
+        <v>5113</v>
       </c>
       <c r="C50" t="n">
-        <v>0.5214534727809064</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>1325223616105HRHT0</t>
+          <t>1325216814085TURP0</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>1132</v>
+        <v>1000</v>
       </c>
       <c r="C51" t="n">
-        <v>0.507634754625905</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>1425118916008QRBT0</t>
+          <t>1325216814085TURS0</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>8509</v>
+        <v>300</v>
       </c>
       <c r="C52" t="n">
-        <v>0.5241351568785197</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>1D25212812074FXC10</t>
+          <t>1325217413077TUSP0</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>28177</v>
+        <v>5703</v>
       </c>
       <c r="C53" t="n">
-        <v>0.4980825958702065</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>1D25212812086FXPC0</t>
+          <t>1325217415081HUTR0</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>24623</v>
+        <v>1524</v>
       </c>
       <c r="C54" t="n">
-        <v>0.4858541163850899</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>1D25213812090FXPC0</t>
+          <t>1325217514082HURL2</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>27462</v>
+        <v>2362</v>
       </c>
       <c r="C55" t="n">
-        <v>0.4945427728613569</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>1D25215013008SXC11</t>
+          <t>1325217514082HURP0</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>1575</v>
+        <v>421</v>
       </c>
       <c r="C56" t="n">
-        <v>0.4863904532046125</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
+          <t>1325217514082TTMX0</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>6492</v>
+      </c>
+      <c r="C57" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>1325217514082TUTR0</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>2515</v>
+      </c>
+      <c r="C58" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>1325217514082TVECH</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>3200</v>
+      </c>
+      <c r="C59" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>1325217514086VURL0</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>1273</v>
+      </c>
+      <c r="C60" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>1325217613082TUNE0</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>4202</v>
+      </c>
+      <c r="C61" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>1325217613082TUNE2</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>2618</v>
+      </c>
+      <c r="C62" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>1325217614084HURL1</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>1379</v>
+      </c>
+      <c r="C63" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>1325217614084HURL2</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>1295</v>
+      </c>
+      <c r="C64" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>1325218414082HUSP0</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>1386</v>
+      </c>
+      <c r="C65" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>1325218414086VURL0</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>909</v>
+      </c>
+      <c r="C66" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>1325218415084TTMX0</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>1557</v>
+      </c>
+      <c r="C67" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>1325218416086VURL0</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>2500</v>
+      </c>
+      <c r="C68" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>1325218514086HURL0</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>2500</v>
+      </c>
+      <c r="C69" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>1325218515088HTMX0</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>12000</v>
+      </c>
+      <c r="C70" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>1325218515088HURP0</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>456</v>
+      </c>
+      <c r="C71" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>1325218515088HUTR0</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>4924</v>
+      </c>
+      <c r="C72" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>1325218515088TURL0</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>2136</v>
+      </c>
+      <c r="C73" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>1325218515088TURS0</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>300</v>
+      </c>
+      <c r="C74" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>1325218614088HURL0</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>1034</v>
+      </c>
+      <c r="C75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>1325218614092VURL0</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>11</v>
+      </c>
+      <c r="C76" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>1325218615089HURL0</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>1314</v>
+      </c>
+      <c r="C77" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>1325219316087VURP0</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>609</v>
+      </c>
+      <c r="C78" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>1325219316087VUTR0</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>7000</v>
+      </c>
+      <c r="C79" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>1325219415088VURL1</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C80" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>1325219416089HRHE0</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>17000</v>
+      </c>
+      <c r="C81" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>1325219515091VZEP0</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>951</v>
+      </c>
+      <c r="C82" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>1325219515095VLHP0</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>12</v>
+      </c>
+      <c r="C83" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>1325220316091VURL1</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>2778</v>
+      </c>
+      <c r="C84" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>1325220416092VURL0</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>909</v>
+      </c>
+      <c r="C85" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>1325220416092VURP0</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>536</v>
+      </c>
+      <c r="C86" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>1325220515094VTMX0</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>651</v>
+      </c>
+      <c r="C87" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>1325220515094VUTR0</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>6098</v>
+      </c>
+      <c r="C88" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>1325220515094VZEP0</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>558</v>
+      </c>
+      <c r="C89" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>1325220516095HTMX0</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C90" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>1325220516095HUTR0</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>1586</v>
+      </c>
+      <c r="C91" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>1325221117091YLEV0</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>20</v>
+      </c>
+      <c r="C92" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>1325221217095YLEV0</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>40</v>
+      </c>
+      <c r="C93" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>1325221317098VUX10</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>102</v>
+      </c>
+      <c r="C94" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>1325221416095VURL0</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>12000</v>
+      </c>
+      <c r="C95" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>1325221416095VURS0</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>300</v>
+      </c>
+      <c r="C96" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>1325221417100HURL1</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>17000</v>
+      </c>
+      <c r="C97" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>1325221417100HURS0</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>300</v>
+      </c>
+      <c r="C98" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>1325221715100SRHT0</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>19000</v>
+      </c>
+      <c r="C99" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>1325221715100SRXT0</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>4000</v>
+      </c>
+      <c r="C100" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>1325222117094YLEV0</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>1003</v>
+      </c>
+      <c r="C101" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>1325222217098VUX10</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>26</v>
+      </c>
+      <c r="C102" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>1325222317101VUX10</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>456</v>
+      </c>
+      <c r="C103" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>1325222417099HURL0</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>2500</v>
+      </c>
+      <c r="C104" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>1325223418103HRHP0</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>2500</v>
+      </c>
+      <c r="C105" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>1325223517104HRHT0</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>8000</v>
+      </c>
+      <c r="C106" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>1325223517104HRPG0</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>579</v>
+      </c>
+      <c r="C107" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>1325223616105HRHT0</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>2847</v>
+      </c>
+      <c r="C108" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>1325223715105SRXT0</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>3274</v>
+      </c>
+      <c r="C109" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>1325223916120QRAB0</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>1113</v>
+      </c>
+      <c r="C110" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>1325226517112HRHT0</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>3325</v>
+      </c>
+      <c r="C111" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>1425118916008QRBT0</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>9000</v>
+      </c>
+      <c r="C112" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>1D25114012008QSTL0</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C113" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>1D25115013008QXPC0</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C114" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>1D25212812074FXC10</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>30360</v>
+      </c>
+      <c r="C115" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>1D25212812086FXPC0</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>25800</v>
+      </c>
+      <c r="C116" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>1D25213812090FXPC0</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>29040</v>
+      </c>
+      <c r="C117" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>1D25214012006QXC10</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>300</v>
+      </c>
+      <c r="C118" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>1D25214012008QSTL0</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C119" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>1D25215013008SXC11</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>26000</v>
+      </c>
+      <c r="C120" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
           <t>1D25215Z13008QXPC0</t>
         </is>
       </c>
-      <c r="B57" t="n">
-        <v>1093</v>
-      </c>
-      <c r="C57" t="n">
-        <v>0.5044194153928667</v>
+      <c r="B121" t="n">
+        <v>5148</v>
+      </c>
+      <c r="C121" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added April, may and june building pde and updated the pipeline as building must follow the initial curing schedule & improved GT allocation.
</commit_message>
<xml_diff>
--- a/load_demand.xlsx
+++ b/load_demand.xlsx
@@ -443,7 +443,7 @@
         <v>1703</v>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>0.5045669080182354</v>
       </c>
     </row>
     <row r="3">
@@ -456,7 +456,7 @@
         <v>5668</v>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>0.5151997854652722</v>
       </c>
     </row>
     <row r="4">
@@ -469,7 +469,7 @@
         <v>1991</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>0.5041324751944221</v>
       </c>
     </row>
     <row r="5">
@@ -482,7 +482,7 @@
         <v>1787</v>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>0.504792169482435</v>
       </c>
     </row>
     <row r="6">
@@ -495,7 +495,7 @@
         <v>5200</v>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>0.4306114239742558</v>
       </c>
     </row>
     <row r="7">
@@ -508,7 +508,7 @@
         <v>65500</v>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>0.6340842048806651</v>
       </c>
     </row>
     <row r="8">
@@ -521,7 +521,7 @@
         <v>346</v>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
+        <v>0.3342611960311075</v>
       </c>
     </row>
     <row r="9">
@@ -534,7 +534,7 @@
         <v>2900</v>
       </c>
       <c r="C9" t="n">
-        <v>1</v>
+        <v>0.5077768838830786</v>
       </c>
     </row>
     <row r="10">
@@ -547,7 +547,7 @@
         <v>242</v>
       </c>
       <c r="C10" t="n">
-        <v>1</v>
+        <v>0.3339823008849557</v>
       </c>
     </row>
     <row r="11">
@@ -560,7 +560,7 @@
         <v>615</v>
       </c>
       <c r="C11" t="n">
-        <v>1</v>
+        <v>0.3349825690533655</v>
       </c>
     </row>
     <row r="12">
@@ -573,7 +573,7 @@
         <v>14167</v>
       </c>
       <c r="C12" t="n">
-        <v>1</v>
+        <v>0.5205604719764012</v>
       </c>
     </row>
     <row r="13">
@@ -586,7 +586,7 @@
         <v>1320</v>
       </c>
       <c r="C13" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="14">
@@ -599,7 +599,7 @@
         <v>93</v>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>0.3335827299544114</v>
       </c>
     </row>
     <row r="15">
@@ -612,7 +612,7 @@
         <v>1079</v>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>0.5028935371413248</v>
       </c>
     </row>
     <row r="16">
@@ -625,7 +625,7 @@
         <v>200</v>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>0.4172030034861893</v>
       </c>
     </row>
     <row r="17">
@@ -638,7 +638,7 @@
         <v>11420</v>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>0.5080986859747921</v>
       </c>
     </row>
     <row r="18">
@@ -651,7 +651,7 @@
         <v>711</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>0.3352400107267364</v>
       </c>
     </row>
     <row r="19">
@@ -664,7 +664,7 @@
         <v>148</v>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>0.5003968892464468</v>
       </c>
     </row>
     <row r="20">
@@ -677,7 +677,7 @@
         <v>20000</v>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>0.553633681952266</v>
       </c>
     </row>
     <row r="21">
@@ -690,7 +690,7 @@
         <v>12000</v>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>0.5321802091713597</v>
       </c>
     </row>
     <row r="22">
@@ -703,7 +703,7 @@
         <v>5889.000000000001</v>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>0.5001582193617592</v>
       </c>
     </row>
     <row r="23">
@@ -716,7 +716,7 @@
         <v>4000</v>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>0.5107267363904532</v>
       </c>
     </row>
     <row r="24">
@@ -729,7 +729,7 @@
         <v>4569</v>
       </c>
       <c r="C24" t="n">
-        <v>1</v>
+        <v>0.5122526146419952</v>
       </c>
     </row>
     <row r="25">
@@ -742,7 +742,7 @@
         <v>3188</v>
       </c>
       <c r="C25" t="n">
-        <v>1</v>
+        <v>0.5085492089031912</v>
       </c>
     </row>
     <row r="26">
@@ -755,7 +755,7 @@
         <v>4770</v>
       </c>
       <c r="C26" t="n">
-        <v>1</v>
+        <v>0.5127916331456155</v>
       </c>
     </row>
     <row r="27">
@@ -768,7 +768,7 @@
         <v>6500</v>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>0.5174309466344864</v>
       </c>
     </row>
     <row r="28">
@@ -781,7 +781,7 @@
         <v>900</v>
       </c>
       <c r="C28" t="n">
-        <v>1</v>
+        <v>0.502413515687852</v>
       </c>
     </row>
     <row r="29">
@@ -794,7 +794,7 @@
         <v>752</v>
       </c>
       <c r="C29" t="n">
-        <v>1</v>
+        <v>0.5020166264414052</v>
       </c>
     </row>
     <row r="30">
@@ -807,7 +807,7 @@
         <v>8500</v>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
+        <v>0.4394609814963797</v>
       </c>
     </row>
     <row r="31">
@@ -820,7 +820,7 @@
         <v>6000</v>
       </c>
       <c r="C31" t="n">
-        <v>1</v>
+        <v>0.5160901045856798</v>
       </c>
     </row>
     <row r="32">
@@ -833,7 +833,7 @@
         <v>289</v>
       </c>
       <c r="C32" t="n">
-        <v>1</v>
+        <v>0.5007750067042103</v>
       </c>
     </row>
     <row r="33">
@@ -846,7 +846,7 @@
         <v>27000</v>
       </c>
       <c r="C33" t="n">
-        <v>1</v>
+        <v>0.5724054706355591</v>
       </c>
     </row>
     <row r="34">
@@ -859,7 +859,7 @@
         <v>2900</v>
       </c>
       <c r="C34" t="n">
-        <v>1</v>
+        <v>0.5077768838830786</v>
       </c>
     </row>
     <row r="35">
@@ -872,7 +872,7 @@
         <v>74580</v>
       </c>
       <c r="C35" t="n">
-        <v>1</v>
+        <v>0.6166666666666667</v>
       </c>
     </row>
     <row r="36">
@@ -885,7 +885,7 @@
         <v>7747</v>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>0.5207750067042103</v>
       </c>
     </row>
     <row r="37">
@@ -898,7 +898,7 @@
         <v>4239</v>
       </c>
       <c r="C37" t="n">
-        <v>1</v>
+        <v>0.5113676588897828</v>
       </c>
     </row>
     <row r="38">
@@ -911,7 +911,7 @@
         <v>9200</v>
       </c>
       <c r="C38" t="n">
-        <v>1</v>
+        <v>0.5246714936980423</v>
       </c>
     </row>
     <row r="39">
@@ -924,7 +924,7 @@
         <v>10000</v>
       </c>
       <c r="C39" t="n">
-        <v>1</v>
+        <v>0.526816840976133</v>
       </c>
     </row>
     <row r="40">
@@ -937,7 +937,7 @@
         <v>12000</v>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>0.5321802091713597</v>
       </c>
     </row>
     <row r="41">
@@ -950,7 +950,7 @@
         <v>3005</v>
       </c>
       <c r="C41" t="n">
-        <v>1</v>
+        <v>0.5080584607133279</v>
       </c>
     </row>
     <row r="42">
@@ -963,7 +963,7 @@
         <v>5318</v>
       </c>
       <c r="C42" t="n">
-        <v>1</v>
+        <v>0.5142611960311075</v>
       </c>
     </row>
     <row r="43">
@@ -976,7 +976,7 @@
         <v>6634</v>
       </c>
       <c r="C43" t="n">
-        <v>1</v>
+        <v>0.5177902923035667</v>
       </c>
     </row>
     <row r="44">
@@ -989,7 +989,7 @@
         <v>5866</v>
       </c>
       <c r="C44" t="n">
-        <v>1</v>
+        <v>0.5157307589165996</v>
       </c>
     </row>
     <row r="45">
@@ -1002,7 +1002,7 @@
         <v>290</v>
       </c>
       <c r="C45" t="n">
-        <v>1</v>
+        <v>0.3341110217216412</v>
       </c>
     </row>
     <row r="46">
@@ -1015,7 +1015,7 @@
         <v>4000</v>
       </c>
       <c r="C46" t="n">
-        <v>1</v>
+        <v>0.5107267363904532</v>
       </c>
     </row>
     <row r="47">
@@ -1028,7 +1028,7 @@
         <v>14000</v>
       </c>
       <c r="C47" t="n">
-        <v>1</v>
+        <v>0.5375435773665862</v>
       </c>
     </row>
     <row r="48">
@@ -1041,7 +1041,7 @@
         <v>6076</v>
       </c>
       <c r="C48" t="n">
-        <v>1</v>
+        <v>0.5162939125770984</v>
       </c>
     </row>
     <row r="49">
@@ -1054,7 +1054,7 @@
         <v>5181</v>
       </c>
       <c r="C49" t="n">
-        <v>1</v>
+        <v>0.5138938053097345</v>
       </c>
     </row>
     <row r="50">
@@ -1067,7 +1067,7 @@
         <v>5113</v>
       </c>
       <c r="C50" t="n">
-        <v>1</v>
+        <v>0.5137114507910968</v>
       </c>
     </row>
     <row r="51">
@@ -1080,7 +1080,7 @@
         <v>1000</v>
       </c>
       <c r="C51" t="n">
-        <v>1</v>
+        <v>0.41934835076428</v>
       </c>
     </row>
     <row r="52">
@@ -1093,7 +1093,7 @@
         <v>300</v>
       </c>
       <c r="C52" t="n">
-        <v>1</v>
+        <v>0.500804505229284</v>
       </c>
     </row>
     <row r="53">
@@ -1106,7 +1106,7 @@
         <v>5703</v>
       </c>
       <c r="C53" t="n">
-        <v>1</v>
+        <v>0.5152936444086886</v>
       </c>
     </row>
     <row r="54">
@@ -1119,7 +1119,7 @@
         <v>1524</v>
       </c>
       <c r="C54" t="n">
-        <v>1</v>
+        <v>0.5040868865647626</v>
       </c>
     </row>
     <row r="55">
@@ -1132,7 +1132,7 @@
         <v>2362</v>
       </c>
       <c r="C55" t="n">
-        <v>1</v>
+        <v>0.3396674711718959</v>
       </c>
     </row>
     <row r="56">
@@ -1145,7 +1145,7 @@
         <v>421</v>
       </c>
       <c r="C56" t="n">
-        <v>1</v>
+        <v>0.5011289890050952</v>
       </c>
     </row>
     <row r="57">
@@ -1158,7 +1158,7 @@
         <v>6492</v>
       </c>
       <c r="C57" t="n">
-        <v>1</v>
+        <v>0.5174094931617056</v>
       </c>
     </row>
     <row r="58">
@@ -1171,7 +1171,7 @@
         <v>2515</v>
       </c>
       <c r="C58" t="n">
-        <v>1</v>
+        <v>0.5067444355054974</v>
       </c>
     </row>
     <row r="59">
@@ -1184,7 +1184,7 @@
         <v>3200</v>
       </c>
       <c r="C59" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="60">
@@ -1197,7 +1197,7 @@
         <v>1273</v>
       </c>
       <c r="C60" t="n">
-        <v>1</v>
+        <v>0.336747117189595</v>
       </c>
     </row>
     <row r="61">
@@ -1210,7 +1210,7 @@
         <v>4202</v>
       </c>
       <c r="C61" t="n">
-        <v>1</v>
+        <v>0.3446017699115044</v>
       </c>
     </row>
     <row r="62">
@@ -1223,7 +1223,7 @@
         <v>2618</v>
       </c>
       <c r="C62" t="n">
-        <v>1</v>
+        <v>0.3403539823008849</v>
       </c>
     </row>
     <row r="63">
@@ -1236,7 +1236,7 @@
         <v>1379</v>
       </c>
       <c r="C63" t="n">
-        <v>1</v>
+        <v>0.5036980423706088</v>
       </c>
     </row>
     <row r="64">
@@ -1249,7 +1249,7 @@
         <v>1295</v>
       </c>
       <c r="C64" t="n">
-        <v>1</v>
+        <v>0.3368061142397425</v>
       </c>
     </row>
     <row r="65">
@@ -1262,7 +1262,7 @@
         <v>1386</v>
       </c>
       <c r="C65" t="n">
-        <v>1</v>
+        <v>0.3370501474926254</v>
       </c>
     </row>
     <row r="66">
@@ -1275,7 +1275,7 @@
         <v>909</v>
       </c>
       <c r="C66" t="n">
-        <v>1</v>
+        <v>0.3357709841780638</v>
       </c>
     </row>
     <row r="67">
@@ -1288,7 +1288,7 @@
         <v>1557</v>
       </c>
       <c r="C67" t="n">
-        <v>1</v>
+        <v>0.5041753821399839</v>
       </c>
     </row>
     <row r="68">
@@ -1301,7 +1301,7 @@
         <v>2500</v>
       </c>
       <c r="C68" t="n">
-        <v>1</v>
+        <v>0.4233708769106999</v>
       </c>
     </row>
     <row r="69">
@@ -1314,7 +1314,7 @@
         <v>2500</v>
       </c>
       <c r="C69" t="n">
-        <v>1</v>
+        <v>0.5067042102440332</v>
       </c>
     </row>
     <row r="70">
@@ -1327,7 +1327,7 @@
         <v>12000</v>
       </c>
       <c r="C70" t="n">
-        <v>1</v>
+        <v>0.5321802091713597</v>
       </c>
     </row>
     <row r="71">
@@ -1340,7 +1340,7 @@
         <v>456</v>
       </c>
       <c r="C71" t="n">
-        <v>1</v>
+        <v>0.5012228479485117</v>
       </c>
     </row>
     <row r="72">
@@ -1353,7 +1353,7 @@
         <v>4924</v>
       </c>
       <c r="C72" t="n">
-        <v>1</v>
+        <v>0.5132046124966478</v>
       </c>
     </row>
     <row r="73">
@@ -1366,7 +1366,7 @@
         <v>2136</v>
       </c>
       <c r="C73" t="n">
-        <v>1</v>
+        <v>0.505728077232502</v>
       </c>
     </row>
     <row r="74">
@@ -1379,7 +1379,7 @@
         <v>300</v>
       </c>
       <c r="C74" t="n">
-        <v>1</v>
+        <v>0.500804505229284</v>
       </c>
     </row>
     <row r="75">
@@ -1392,7 +1392,7 @@
         <v>1034</v>
       </c>
       <c r="C75" t="n">
-        <v>1</v>
+        <v>0.5027728613569321</v>
       </c>
     </row>
     <row r="76">
@@ -1405,7 +1405,7 @@
         <v>11</v>
       </c>
       <c r="C76" t="n">
-        <v>1</v>
+        <v>0.333362831858407</v>
       </c>
     </row>
     <row r="77">
@@ -1418,7 +1418,7 @@
         <v>1314</v>
       </c>
       <c r="C77" t="n">
-        <v>1</v>
+        <v>0.5035237329042639</v>
       </c>
     </row>
     <row r="78">
@@ -1431,7 +1431,7 @@
         <v>609</v>
       </c>
       <c r="C78" t="n">
-        <v>1</v>
+        <v>0.5016331456154465</v>
       </c>
     </row>
     <row r="79">
@@ -1444,7 +1444,7 @@
         <v>7000</v>
       </c>
       <c r="C79" t="n">
-        <v>1</v>
+        <v>0.5187717886832931</v>
       </c>
     </row>
     <row r="80">
@@ -1457,7 +1457,7 @@
         <v>2000</v>
       </c>
       <c r="C80" t="n">
-        <v>1</v>
+        <v>0.5053633681952266</v>
       </c>
     </row>
     <row r="81">
@@ -1470,7 +1470,7 @@
         <v>17000</v>
       </c>
       <c r="C81" t="n">
-        <v>1</v>
+        <v>0.5134084204880665</v>
       </c>
     </row>
     <row r="82">
@@ -1483,7 +1483,7 @@
         <v>951</v>
       </c>
       <c r="C82" t="n">
-        <v>1</v>
+        <v>0.3358836149101636</v>
       </c>
     </row>
     <row r="83">
@@ -1496,7 +1496,7 @@
         <v>12</v>
       </c>
       <c r="C83" t="n">
-        <v>1</v>
+        <v>0.3333655135425047</v>
       </c>
     </row>
     <row r="84">
@@ -1509,7 +1509,7 @@
         <v>2778</v>
       </c>
       <c r="C84" t="n">
-        <v>1</v>
+        <v>0.505374094931617</v>
       </c>
     </row>
     <row r="85">
@@ -1522,7 +1522,7 @@
         <v>909</v>
       </c>
       <c r="C85" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="86">
@@ -1535,7 +1535,7 @@
         <v>536</v>
       </c>
       <c r="C86" t="n">
-        <v>1</v>
+        <v>0.5014373826763208</v>
       </c>
     </row>
     <row r="87">
@@ -1548,7 +1548,7 @@
         <v>651</v>
       </c>
       <c r="C87" t="n">
-        <v>1</v>
+        <v>0.5017457763475462</v>
       </c>
     </row>
     <row r="88">
@@ -1561,7 +1561,7 @@
         <v>6098</v>
       </c>
       <c r="C88" t="n">
-        <v>1</v>
+        <v>0.5163529096272459</v>
       </c>
     </row>
     <row r="89">
@@ -1574,7 +1574,7 @@
         <v>558</v>
       </c>
       <c r="C89" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="90">
@@ -1587,7 +1587,7 @@
         <v>5000</v>
       </c>
       <c r="C90" t="n">
-        <v>1</v>
+        <v>0.5134084204880665</v>
       </c>
     </row>
     <row r="91">
@@ -1600,7 +1600,7 @@
         <v>1586</v>
       </c>
       <c r="C91" t="n">
-        <v>1</v>
+        <v>0.5042531509788147</v>
       </c>
     </row>
     <row r="92">
@@ -1613,7 +1613,7 @@
         <v>20</v>
       </c>
       <c r="C92" t="n">
-        <v>1</v>
+        <v>0.3333869670152856</v>
       </c>
     </row>
     <row r="93">
@@ -1626,7 +1626,7 @@
         <v>40</v>
       </c>
       <c r="C93" t="n">
-        <v>1</v>
+        <v>0.3334406006972379</v>
       </c>
     </row>
     <row r="94">
@@ -1639,7 +1639,7 @@
         <v>102</v>
       </c>
       <c r="C94" t="n">
-        <v>1</v>
+        <v>0.5000107267363905</v>
       </c>
     </row>
     <row r="95">
@@ -1652,7 +1652,7 @@
         <v>12000</v>
       </c>
       <c r="C95" t="n">
-        <v>1</v>
+        <v>0.5321802091713597</v>
       </c>
     </row>
     <row r="96">
@@ -1665,7 +1665,7 @@
         <v>300</v>
       </c>
       <c r="C96" t="n">
-        <v>1</v>
+        <v>0.500804505229284</v>
       </c>
     </row>
     <row r="97">
@@ -1678,7 +1678,7 @@
         <v>17000</v>
       </c>
       <c r="C97" t="n">
-        <v>1</v>
+        <v>0.5455886296594261</v>
       </c>
     </row>
     <row r="98">
@@ -1691,7 +1691,7 @@
         <v>300</v>
       </c>
       <c r="C98" t="n">
-        <v>1</v>
+        <v>0.500804505229284</v>
       </c>
     </row>
     <row r="99">
@@ -1704,7 +1704,7 @@
         <v>19000</v>
       </c>
       <c r="C99" t="n">
-        <v>1</v>
+        <v>0.5509519978546528</v>
       </c>
     </row>
     <row r="100">
@@ -1717,7 +1717,7 @@
         <v>4000</v>
       </c>
       <c r="C100" t="n">
-        <v>1</v>
+        <v>0.5107267363904532</v>
       </c>
     </row>
     <row r="101">
@@ -1730,7 +1730,7 @@
         <v>1003</v>
       </c>
       <c r="C101" t="n">
-        <v>1</v>
+        <v>0.3360230624832394</v>
       </c>
     </row>
     <row r="102">
@@ -1743,7 +1743,7 @@
         <v>26</v>
       </c>
       <c r="C102" t="n">
-        <v>1</v>
+        <v>0.3334030571198713</v>
       </c>
     </row>
     <row r="103">
@@ -1756,7 +1756,7 @@
         <v>456</v>
       </c>
       <c r="C103" t="n">
-        <v>1</v>
+        <v>0.334556181281845</v>
       </c>
     </row>
     <row r="104">
@@ -1769,7 +1769,7 @@
         <v>2500</v>
       </c>
       <c r="C104" t="n">
-        <v>1</v>
+        <v>0.5067042102440332</v>
       </c>
     </row>
     <row r="105">
@@ -1782,7 +1782,7 @@
         <v>2500</v>
       </c>
       <c r="C105" t="n">
-        <v>1</v>
+        <v>0.5067042102440332</v>
       </c>
     </row>
     <row r="106">
@@ -1795,7 +1795,7 @@
         <v>8000</v>
       </c>
       <c r="C106" t="n">
-        <v>1</v>
+        <v>0.5214534727809064</v>
       </c>
     </row>
     <row r="107">
@@ -1808,7 +1808,7 @@
         <v>579</v>
       </c>
       <c r="C107" t="n">
-        <v>1</v>
+        <v>0.5015526950925181</v>
       </c>
     </row>
     <row r="108">
@@ -1821,7 +1821,7 @@
         <v>2847</v>
       </c>
       <c r="C108" t="n">
-        <v>1</v>
+        <v>0.507634754625905</v>
       </c>
     </row>
     <row r="109">
@@ -1834,7 +1834,7 @@
         <v>3274</v>
       </c>
       <c r="C109" t="n">
-        <v>1</v>
+        <v>0.508779833735586</v>
       </c>
     </row>
     <row r="110">
@@ -1847,7 +1847,7 @@
         <v>1113</v>
       </c>
       <c r="C110" t="n">
-        <v>1</v>
+        <v>0.3363180477339769</v>
       </c>
     </row>
     <row r="111">
@@ -1860,7 +1860,7 @@
         <v>3325</v>
       </c>
       <c r="C111" t="n">
-        <v>1</v>
+        <v>0.5053633681952266</v>
       </c>
     </row>
     <row r="112">
@@ -1873,7 +1873,7 @@
         <v>9000</v>
       </c>
       <c r="C112" t="n">
-        <v>1</v>
+        <v>0.5241351568785197</v>
       </c>
     </row>
     <row r="113">
@@ -1886,7 +1886,7 @@
         <v>3000</v>
       </c>
       <c r="C113" t="n">
-        <v>1</v>
+        <v>0.5080450522928399</v>
       </c>
     </row>
     <row r="114">
@@ -1899,7 +1899,7 @@
         <v>1500</v>
       </c>
       <c r="C114" t="n">
-        <v>1</v>
+        <v>0.50402252614642</v>
       </c>
     </row>
     <row r="115">
@@ -1912,7 +1912,7 @@
         <v>30360</v>
       </c>
       <c r="C115" t="n">
-        <v>1</v>
+        <v>0.4980825958702065</v>
       </c>
     </row>
     <row r="116">
@@ -1925,7 +1925,7 @@
         <v>25800</v>
       </c>
       <c r="C116" t="n">
-        <v>1</v>
+        <v>0.4858541163850899</v>
       </c>
     </row>
     <row r="117">
@@ -1938,7 +1938,7 @@
         <v>29040</v>
       </c>
       <c r="C117" t="n">
-        <v>1</v>
+        <v>0.4945427728613569</v>
       </c>
     </row>
     <row r="118">
@@ -1951,7 +1951,7 @@
         <v>300</v>
       </c>
       <c r="C118" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="119">
@@ -1964,7 +1964,7 @@
         <v>3000</v>
       </c>
       <c r="C119" t="n">
-        <v>1</v>
+        <v>0.5080450522928399</v>
       </c>
     </row>
     <row r="120">
@@ -1977,7 +1977,7 @@
         <v>26000</v>
       </c>
       <c r="C120" t="n">
-        <v>1</v>
+        <v>0.4863904532046125</v>
       </c>
     </row>
     <row r="121">
@@ -1990,7 +1990,7 @@
         <v>5148</v>
       </c>
       <c r="C121" t="n">
-        <v>1</v>
+        <v>0.5044194153928667</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated building logic- building generates the exact output planned by curing1
</commit_message>
<xml_diff>
--- a/load_demand.xlsx
+++ b/load_demand.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C121"/>
+  <dimension ref="A1:C98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -440,7 +440,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1703</v>
+        <v>532</v>
       </c>
       <c r="C2" t="n">
         <v>0.5045669080182354</v>
@@ -453,7 +453,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5668</v>
+        <v>1512</v>
       </c>
       <c r="C3" t="n">
         <v>0.5151997854652722</v>
@@ -466,7 +466,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1991</v>
+        <v>104</v>
       </c>
       <c r="C4" t="n">
         <v>0.5041324751944221</v>
@@ -479,7 +479,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1787</v>
+        <v>873</v>
       </c>
       <c r="C5" t="n">
         <v>0.504792169482435</v>
@@ -492,7 +492,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5200</v>
+        <v>3577</v>
       </c>
       <c r="C6" t="n">
         <v>0.4306114239742558</v>
@@ -505,7 +505,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>65500</v>
+        <v>54776</v>
       </c>
       <c r="C7" t="n">
         <v>0.6340842048806651</v>
@@ -518,7 +518,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>346</v>
+        <v>70</v>
       </c>
       <c r="C8" t="n">
         <v>0.3342611960311075</v>
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2900</v>
+        <v>365</v>
       </c>
       <c r="C9" t="n">
         <v>0.5077768838830786</v>
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>242</v>
+        <v>36</v>
       </c>
       <c r="C10" t="n">
         <v>0.3339823008849557</v>
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>615</v>
+        <v>375</v>
       </c>
       <c r="C11" t="n">
         <v>0.3349825690533655</v>
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>14167</v>
+        <v>3408</v>
       </c>
       <c r="C12" t="n">
         <v>0.5205604719764012</v>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1320</v>
+        <v>68</v>
       </c>
       <c r="C13" t="n">
         <v>0.5</v>
@@ -592,1404 +592,1105 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1225222615008RXC10</t>
+          <t>1225222716121NXC11</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>93</v>
+        <v>1</v>
       </c>
       <c r="C14" t="n">
-        <v>0.3335827299544114</v>
+        <v>0.4172030034861893</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1225222716121MXC11</t>
+          <t>1225223516121PSKP0</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1079</v>
+        <v>11420</v>
       </c>
       <c r="C15" t="n">
-        <v>0.5028935371413248</v>
+        <v>0.5080986859747921</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1225222716121NXC11</t>
+          <t>1325114812074TUHL0</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>200</v>
+        <v>14986</v>
       </c>
       <c r="C16" t="n">
-        <v>0.4172030034861893</v>
+        <v>0.553633681952266</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1225223516121PSKP0</t>
+          <t>1325119015008SRBT0</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>11420</v>
+        <v>3263</v>
       </c>
       <c r="C17" t="n">
-        <v>0.5080986859747921</v>
+        <v>0.5321802091713597</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1225223516121RBVN0</t>
+          <t>1325119815106QBRQ0</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>711</v>
+        <v>561</v>
       </c>
       <c r="C18" t="n">
-        <v>0.3352400107267364</v>
+        <v>0.5001582193617592</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1325114613071TTMX0</t>
+          <t>1325121715100SBRT0</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>148</v>
+        <v>1519</v>
       </c>
       <c r="C19" t="n">
-        <v>0.5003968892464468</v>
+        <v>0.5107267363904532</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1325114812074TUHL0</t>
+          <t>1325121715100SRBT0</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>20000</v>
+        <v>1228</v>
       </c>
       <c r="C20" t="n">
-        <v>0.553633681952266</v>
+        <v>0.5122526146419952</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1325119015008SRBT0</t>
+          <t>1325121715100SRXT0</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>12000</v>
+        <v>700</v>
       </c>
       <c r="C21" t="n">
-        <v>0.5321802091713597</v>
+        <v>0.5085492089031912</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1325119815106QBRQ0</t>
+          <t>1325121715115SLTB0</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>5889.000000000001</v>
+        <v>1342</v>
       </c>
       <c r="C22" t="n">
-        <v>0.5001582193617592</v>
+        <v>0.5127916331456155</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1325121715100SBRT0</t>
+          <t>1325123715105SBRT0</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>4000</v>
+        <v>1252</v>
       </c>
       <c r="C23" t="n">
-        <v>0.5107267363904532</v>
+        <v>0.5174309466344864</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1325121715100SRBT0</t>
+          <t>1325123715105SRXT0</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>4569</v>
+        <v>150</v>
       </c>
       <c r="C24" t="n">
-        <v>0.5122526146419952</v>
+        <v>0.502413515687852</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1325121715100SRXT0</t>
+          <t>1325213612065SULX1</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>3188</v>
+        <v>752</v>
       </c>
       <c r="C25" t="n">
-        <v>0.5085492089031912</v>
+        <v>0.5020166264414052</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1325121715115SLTB0</t>
+          <t>1325213615099MSXT0</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>4770</v>
+        <v>4249</v>
       </c>
       <c r="C26" t="n">
-        <v>0.5127916331456155</v>
+        <v>0.4394609814963797</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1325123715105SBRT0</t>
+          <t>1325214613071TTMX0</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>6500</v>
+        <v>89</v>
       </c>
       <c r="C27" t="n">
-        <v>0.5174309466344864</v>
+        <v>0.5007750067042103</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1325123715105SRXT0</t>
+          <t>1325214812074TUHL0</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>900</v>
+        <v>24182</v>
       </c>
       <c r="C28" t="n">
-        <v>0.502413515687852</v>
+        <v>0.5724054706355591</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1325213612065SULX1</t>
+          <t>1325214813075STMX0</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>752</v>
+        <v>1506</v>
       </c>
       <c r="C29" t="n">
-        <v>0.5020166264414052</v>
+        <v>0.5077768838830786</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1325213615099MSXT0</t>
+          <t>1325214813075SUNE1</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>8500</v>
+        <v>66042</v>
       </c>
       <c r="C30" t="n">
-        <v>0.4394609814963797</v>
+        <v>0.6166666666666667</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1325214612069TUHL0</t>
+          <t>1325215513073TUHL0</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>6000</v>
+        <v>39</v>
       </c>
       <c r="C31" t="n">
-        <v>0.5160901045856798</v>
+        <v>0.5207750067042103</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1325214613071TTMX0</t>
+          <t>1325215613075TTMX0</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>289</v>
+        <v>1418</v>
       </c>
       <c r="C32" t="n">
-        <v>0.5007750067042103</v>
+        <v>0.5113676588897828</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1325214812074TUHL0</t>
+          <t>1325215613075TUHL0</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>27000</v>
+        <v>3888</v>
       </c>
       <c r="C33" t="n">
-        <v>0.5724054706355591</v>
+        <v>0.5246714936980423</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1325214813075STMX0</t>
+          <t>1325215813079STMX0</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2900</v>
+        <v>4671</v>
       </c>
       <c r="C34" t="n">
-        <v>0.5077768838830786</v>
+        <v>0.526816840976133</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1325214813075SUNE1</t>
+          <t>1325215813079SUHL0</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>74580</v>
+        <v>7101</v>
       </c>
       <c r="C35" t="n">
-        <v>0.6166666666666667</v>
+        <v>0.5321802091713597</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>1325215513073TUHL0</t>
+          <t>1325216513077TUHL0</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>7747</v>
+        <v>1679</v>
       </c>
       <c r="C36" t="n">
-        <v>0.5207750067042103</v>
+        <v>0.5080584607133279</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1325215613075TTMX0</t>
+          <t>1325216514079TTMX0</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>4239</v>
+        <v>5305</v>
       </c>
       <c r="C37" t="n">
-        <v>0.5113676588897828</v>
+        <v>0.5142611960311075</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>1325215613075TUHL0</t>
+          <t>1325216614081STMX0</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>9200</v>
+        <v>6451</v>
       </c>
       <c r="C38" t="n">
-        <v>0.5246714936980423</v>
+        <v>0.5177902923035667</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>1325215813079STMX0</t>
+          <t>1325216614081SUTR0</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>10000</v>
+        <v>5866</v>
       </c>
       <c r="C39" t="n">
-        <v>0.526816840976133</v>
+        <v>0.5157307589165996</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>1325215813079SUHL0</t>
+          <t>1325216614081TVECE</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>12000</v>
+        <v>290</v>
       </c>
       <c r="C40" t="n">
-        <v>0.5321802091713597</v>
+        <v>0.3341110217216412</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>1325216513077TUHL0</t>
+          <t>1325216813083TUNE0</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>3005</v>
+        <v>2344</v>
       </c>
       <c r="C41" t="n">
-        <v>0.5080584607133279</v>
+        <v>0.5107267363904532</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>1325216514079TTMX0</t>
+          <t>1325216814085STMX0</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>5318</v>
+        <v>14000</v>
       </c>
       <c r="C42" t="n">
-        <v>0.5142611960311075</v>
+        <v>0.5375435773665862</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>1325216614081STMX0</t>
+          <t>1325216814085SURL0</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>6634</v>
+        <v>427</v>
       </c>
       <c r="C43" t="n">
-        <v>0.5177902923035667</v>
+        <v>0.5162939125770984</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>1325216614081SUTR0</t>
+          <t>1325216814085SUTR0</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>5866</v>
+        <v>4582</v>
       </c>
       <c r="C44" t="n">
-        <v>0.5157307589165996</v>
+        <v>0.5138938053097345</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>1325216614081TVECE</t>
+          <t>1325216814085TURL0</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>290</v>
+        <v>5113</v>
       </c>
       <c r="C45" t="n">
-        <v>0.3341110217216412</v>
+        <v>0.5137114507910968</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>1325216813083TUNE0</t>
+          <t>1325216814085TURS0</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>4000</v>
+        <v>300</v>
       </c>
       <c r="C46" t="n">
-        <v>0.5107267363904532</v>
+        <v>0.500804505229284</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>1325216814085STMX0</t>
+          <t>1325217413077TUSP0</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>14000</v>
+        <v>3263</v>
       </c>
       <c r="C47" t="n">
-        <v>0.5375435773665862</v>
+        <v>0.5152936444086886</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>1325216814085SURL0</t>
+          <t>1325217415081HUTR0</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>6076</v>
+        <v>1524</v>
       </c>
       <c r="C48" t="n">
-        <v>0.5162939125770984</v>
+        <v>0.5040868865647626</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>1325216814085SUTR0</t>
+          <t>1325217514082HURL2</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>5181</v>
+        <v>1868</v>
       </c>
       <c r="C49" t="n">
-        <v>0.5138938053097345</v>
+        <v>0.3396674711718959</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>1325216814085TURL0</t>
+          <t>1325217514082TTMX0</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>5113</v>
+        <v>6492</v>
       </c>
       <c r="C50" t="n">
-        <v>0.5137114507910968</v>
+        <v>0.5174094931617056</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>1325216814085TURP0</t>
+          <t>1325217514082TUTR0</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>1000</v>
+        <v>2515</v>
       </c>
       <c r="C51" t="n">
-        <v>0.41934835076428</v>
+        <v>0.5067444355054974</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>1325216814085TURS0</t>
+          <t>1325217514082TVECH</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>300</v>
+        <v>2124</v>
       </c>
       <c r="C52" t="n">
-        <v>0.500804505229284</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>1325217413077TUSP0</t>
+          <t>1325217613082TUNE0</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>5703</v>
+        <v>2824</v>
       </c>
       <c r="C53" t="n">
-        <v>0.5152936444086886</v>
+        <v>0.3446017699115044</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>1325217415081HUTR0</t>
+          <t>1325217613082TUNE2</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>1524</v>
+        <v>2618</v>
       </c>
       <c r="C54" t="n">
-        <v>0.5040868865647626</v>
+        <v>0.3403539823008849</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>1325217514082HURL2</t>
+          <t>1325217614084HURL2</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>2362</v>
+        <v>895</v>
       </c>
       <c r="C55" t="n">
-        <v>0.3396674711718959</v>
+        <v>0.3368061142397425</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>1325217514082HURP0</t>
+          <t>1325218415084TTMX0</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>421</v>
+        <v>90</v>
       </c>
       <c r="C56" t="n">
-        <v>0.5011289890050952</v>
+        <v>0.5041753821399839</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>1325217514082TTMX0</t>
+          <t>1325218416086VURL0</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>6492</v>
+        <v>2500</v>
       </c>
       <c r="C57" t="n">
-        <v>0.5174094931617056</v>
+        <v>0.4233708769106999</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>1325217514082TUTR0</t>
+          <t>1325218514086HURL0</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>2515</v>
+        <v>2500</v>
       </c>
       <c r="C58" t="n">
-        <v>0.5067444355054974</v>
+        <v>0.5067042102440332</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>1325217514082TVECH</t>
+          <t>1325218515088HTMX0</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>3200</v>
+        <v>11421</v>
       </c>
       <c r="C59" t="n">
-        <v>0.5</v>
+        <v>0.5321802091713597</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>1325217514086VURL0</t>
+          <t>1325218515088HURP0</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>1273</v>
+        <v>456</v>
       </c>
       <c r="C60" t="n">
-        <v>0.336747117189595</v>
+        <v>0.5012228479485117</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>1325217613082TUNE0</t>
+          <t>1325218515088HUTR0</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>4202</v>
+        <v>4924</v>
       </c>
       <c r="C61" t="n">
-        <v>0.3446017699115044</v>
+        <v>0.5132046124966478</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>1325217613082TUNE2</t>
+          <t>1325218515088TURL0</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>2618</v>
+        <v>2136</v>
       </c>
       <c r="C62" t="n">
-        <v>0.3403539823008849</v>
+        <v>0.505728077232502</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>1325217614084HURL1</t>
+          <t>1325218614088HURL0</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>1379</v>
+        <v>676</v>
       </c>
       <c r="C63" t="n">
-        <v>0.5036980423706088</v>
+        <v>0.5027728613569321</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>1325217614084HURL2</t>
+          <t>1325218615089HURL0</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>1295</v>
+        <v>1314</v>
       </c>
       <c r="C64" t="n">
-        <v>0.3368061142397425</v>
+        <v>0.5035237329042639</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>1325218414082HUSP0</t>
+          <t>1325219316087VURP0</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>1386</v>
+        <v>609</v>
       </c>
       <c r="C65" t="n">
-        <v>0.3370501474926254</v>
+        <v>0.5016331456154465</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>1325218414086VURL0</t>
+          <t>1325219316087VUTR0</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>909</v>
+        <v>6044</v>
       </c>
       <c r="C66" t="n">
-        <v>0.3357709841780638</v>
+        <v>0.5187717886832931</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>1325218415084TTMX0</t>
+          <t>1325219415088VURL1</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>1557</v>
+        <v>2000</v>
       </c>
       <c r="C67" t="n">
-        <v>0.5041753821399839</v>
+        <v>0.5053633681952266</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>1325218416086VURL0</t>
+          <t>1325219416089HRHE0</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>2500</v>
+        <v>15404</v>
       </c>
       <c r="C68" t="n">
-        <v>0.4233708769106999</v>
+        <v>0.5134084204880665</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>1325218514086HURL0</t>
+          <t>1325219515091VZEP0</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>2500</v>
+        <v>951</v>
       </c>
       <c r="C69" t="n">
-        <v>0.5067042102440332</v>
+        <v>0.3358836149101636</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>1325218515088HTMX0</t>
+          <t>1325220316091VURL1</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>12000</v>
+        <v>2761</v>
       </c>
       <c r="C70" t="n">
-        <v>0.5321802091713597</v>
+        <v>0.505374094931617</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>1325218515088HURP0</t>
+          <t>1325220416092VURL0</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>456</v>
+        <v>859</v>
       </c>
       <c r="C71" t="n">
-        <v>0.5012228479485117</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>1325218515088HUTR0</t>
+          <t>1325220416092VURP0</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>4924</v>
+        <v>536</v>
       </c>
       <c r="C72" t="n">
-        <v>0.5132046124966478</v>
+        <v>0.5014373826763208</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>1325218515088TURL0</t>
+          <t>1325220515094VTMX0</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>2136</v>
+        <v>651</v>
       </c>
       <c r="C73" t="n">
-        <v>0.505728077232502</v>
+        <v>0.5017457763475462</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>1325218515088TURS0</t>
+          <t>1325220515094VUTR0</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>300</v>
+        <v>6098</v>
       </c>
       <c r="C74" t="n">
-        <v>0.500804505229284</v>
+        <v>0.5163529096272459</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>1325218614088HURL0</t>
+          <t>1325220515094VZEP0</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>1034</v>
+        <v>558</v>
       </c>
       <c r="C75" t="n">
-        <v>0.5027728613569321</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>1325218614092VURL0</t>
+          <t>1325220516095HTMX0</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>11</v>
+        <v>4999</v>
       </c>
       <c r="C76" t="n">
-        <v>0.333362831858407</v>
+        <v>0.5134084204880665</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>1325218615089HURL0</t>
+          <t>1325220516095HUTR0</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>1314</v>
+        <v>742</v>
       </c>
       <c r="C77" t="n">
-        <v>0.5035237329042639</v>
+        <v>0.5042531509788147</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>1325219316087VURP0</t>
+          <t>1325221317098VUX10</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>609</v>
+        <v>102</v>
       </c>
       <c r="C78" t="n">
-        <v>0.5016331456154465</v>
+        <v>0.5000107267363905</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>1325219316087VUTR0</t>
+          <t>1325221416095VURL0</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>7000</v>
+        <v>11230</v>
       </c>
       <c r="C79" t="n">
-        <v>0.5187717886832931</v>
+        <v>0.5321802091713597</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>1325219415088VURL1</t>
+          <t>1325221417100HURL1</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>2000</v>
+        <v>17000</v>
       </c>
       <c r="C80" t="n">
-        <v>0.5053633681952266</v>
+        <v>0.5455886296594261</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>1325219416089HRHE0</t>
+          <t>1325221417100HURS0</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>17000</v>
+        <v>143</v>
       </c>
       <c r="C81" t="n">
-        <v>0.5134084204880665</v>
+        <v>0.500804505229284</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>1325219515091VZEP0</t>
+          <t>1325221715100SRHT0</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>951</v>
+        <v>19000</v>
       </c>
       <c r="C82" t="n">
-        <v>0.3358836149101636</v>
+        <v>0.5509519978546528</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>1325219515095VLHP0</t>
+          <t>1325221715100SRXT0</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>12</v>
+        <v>308</v>
       </c>
       <c r="C83" t="n">
-        <v>0.3333655135425047</v>
+        <v>0.5107267363904532</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>1325220316091VURL1</t>
+          <t>1325222317101VUX10</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>2778</v>
+        <v>456</v>
       </c>
       <c r="C84" t="n">
-        <v>0.505374094931617</v>
+        <v>0.334556181281845</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>1325220416092VURL0</t>
+          <t>1325222417099HURL0</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>909</v>
+        <v>2421</v>
       </c>
       <c r="C85" t="n">
-        <v>0.5</v>
+        <v>0.5067042102440332</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>1325220416092VURP0</t>
+          <t>1325223517104HRHT0</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>536</v>
+        <v>8000</v>
       </c>
       <c r="C86" t="n">
-        <v>0.5014373826763208</v>
+        <v>0.5214534727809064</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>1325220515094VTMX0</t>
+          <t>1325223517104HRPG0</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>651</v>
+        <v>579</v>
       </c>
       <c r="C87" t="n">
-        <v>0.5017457763475462</v>
+        <v>0.5015526950925181</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>1325220515094VUTR0</t>
+          <t>1325223715105SRXT0</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>6098</v>
+        <v>982</v>
       </c>
       <c r="C88" t="n">
-        <v>0.5163529096272459</v>
+        <v>0.508779833735586</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>1325220515094VZEP0</t>
+          <t>1325226517112HRHT0</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>558</v>
+        <v>3325</v>
       </c>
       <c r="C89" t="n">
-        <v>0.5</v>
+        <v>0.5053633681952266</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>1325220516095HTMX0</t>
+          <t>1425118916008QRBT0</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>5000</v>
+        <v>9000</v>
       </c>
       <c r="C90" t="n">
-        <v>0.5134084204880665</v>
+        <v>0.5241351568785197</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>1325220516095HUTR0</t>
+          <t>1D25115013008QXPC0</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>1586</v>
+        <v>471</v>
       </c>
       <c r="C91" t="n">
-        <v>0.5042531509788147</v>
+        <v>0.50402252614642</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>1325221117091YLEV0</t>
+          <t>1D25212812074FXC10</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>20</v>
+        <v>18658</v>
       </c>
       <c r="C92" t="n">
-        <v>0.3333869670152856</v>
+        <v>0.4980825958702065</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>1325221217095YLEV0</t>
+          <t>1D25212812086FXPC0</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>40</v>
+        <v>18100</v>
       </c>
       <c r="C93" t="n">
-        <v>0.3334406006972379</v>
+        <v>0.4858541163850899</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>1325221317098VUX10</t>
+          <t>1D25213812090FXPC0</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>102</v>
+        <v>19334</v>
       </c>
       <c r="C94" t="n">
-        <v>0.5000107267363905</v>
+        <v>0.4945427728613569</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>1325221416095VURL0</t>
+          <t>1D25214012006QXC10</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>12000</v>
+        <v>300</v>
       </c>
       <c r="C95" t="n">
-        <v>0.5321802091713597</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>1325221416095VURS0</t>
+          <t>1D25214012008QSTL0</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>300</v>
+        <v>2206</v>
       </c>
       <c r="C96" t="n">
-        <v>0.500804505229284</v>
+        <v>0.5080450522928399</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>1325221417100HURL1</t>
+          <t>1D25215013008SXC11</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>17000</v>
+        <v>24086</v>
       </c>
       <c r="C97" t="n">
-        <v>0.5455886296594261</v>
+        <v>0.4863904532046125</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>1325221417100HURS0</t>
+          <t>1D25215Z13008QXPC0</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>300</v>
+        <v>2338</v>
       </c>
       <c r="C98" t="n">
-        <v>0.500804505229284</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>1325221715100SRHT0</t>
-        </is>
-      </c>
-      <c r="B99" t="n">
-        <v>19000</v>
-      </c>
-      <c r="C99" t="n">
-        <v>0.5509519978546528</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>1325221715100SRXT0</t>
-        </is>
-      </c>
-      <c r="B100" t="n">
-        <v>4000</v>
-      </c>
-      <c r="C100" t="n">
-        <v>0.5107267363904532</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>1325222117094YLEV0</t>
-        </is>
-      </c>
-      <c r="B101" t="n">
-        <v>1003</v>
-      </c>
-      <c r="C101" t="n">
-        <v>0.3360230624832394</v>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>1325222217098VUX10</t>
-        </is>
-      </c>
-      <c r="B102" t="n">
-        <v>26</v>
-      </c>
-      <c r="C102" t="n">
-        <v>0.3334030571198713</v>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>1325222317101VUX10</t>
-        </is>
-      </c>
-      <c r="B103" t="n">
-        <v>456</v>
-      </c>
-      <c r="C103" t="n">
-        <v>0.334556181281845</v>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>1325222417099HURL0</t>
-        </is>
-      </c>
-      <c r="B104" t="n">
-        <v>2500</v>
-      </c>
-      <c r="C104" t="n">
-        <v>0.5067042102440332</v>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>1325223418103HRHP0</t>
-        </is>
-      </c>
-      <c r="B105" t="n">
-        <v>2500</v>
-      </c>
-      <c r="C105" t="n">
-        <v>0.5067042102440332</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>1325223517104HRHT0</t>
-        </is>
-      </c>
-      <c r="B106" t="n">
-        <v>8000</v>
-      </c>
-      <c r="C106" t="n">
-        <v>0.5214534727809064</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>1325223517104HRPG0</t>
-        </is>
-      </c>
-      <c r="B107" t="n">
-        <v>579</v>
-      </c>
-      <c r="C107" t="n">
-        <v>0.5015526950925181</v>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>1325223616105HRHT0</t>
-        </is>
-      </c>
-      <c r="B108" t="n">
-        <v>2847</v>
-      </c>
-      <c r="C108" t="n">
-        <v>0.507634754625905</v>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>1325223715105SRXT0</t>
-        </is>
-      </c>
-      <c r="B109" t="n">
-        <v>3274</v>
-      </c>
-      <c r="C109" t="n">
-        <v>0.508779833735586</v>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>1325223916120QRAB0</t>
-        </is>
-      </c>
-      <c r="B110" t="n">
-        <v>1113</v>
-      </c>
-      <c r="C110" t="n">
-        <v>0.3363180477339769</v>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>1325226517112HRHT0</t>
-        </is>
-      </c>
-      <c r="B111" t="n">
-        <v>3325</v>
-      </c>
-      <c r="C111" t="n">
-        <v>0.5053633681952266</v>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>1425118916008QRBT0</t>
-        </is>
-      </c>
-      <c r="B112" t="n">
-        <v>9000</v>
-      </c>
-      <c r="C112" t="n">
-        <v>0.5241351568785197</v>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>1D25114012008QSTL0</t>
-        </is>
-      </c>
-      <c r="B113" t="n">
-        <v>3000</v>
-      </c>
-      <c r="C113" t="n">
-        <v>0.5080450522928399</v>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>1D25115013008QXPC0</t>
-        </is>
-      </c>
-      <c r="B114" t="n">
-        <v>1500</v>
-      </c>
-      <c r="C114" t="n">
-        <v>0.50402252614642</v>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>1D25212812074FXC10</t>
-        </is>
-      </c>
-      <c r="B115" t="n">
-        <v>30360</v>
-      </c>
-      <c r="C115" t="n">
-        <v>0.4980825958702065</v>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>1D25212812086FXPC0</t>
-        </is>
-      </c>
-      <c r="B116" t="n">
-        <v>25800</v>
-      </c>
-      <c r="C116" t="n">
-        <v>0.4858541163850899</v>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>1D25213812090FXPC0</t>
-        </is>
-      </c>
-      <c r="B117" t="n">
-        <v>29040</v>
-      </c>
-      <c r="C117" t="n">
-        <v>0.4945427728613569</v>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>1D25214012006QXC10</t>
-        </is>
-      </c>
-      <c r="B118" t="n">
-        <v>300</v>
-      </c>
-      <c r="C118" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>1D25214012008QSTL0</t>
-        </is>
-      </c>
-      <c r="B119" t="n">
-        <v>3000</v>
-      </c>
-      <c r="C119" t="n">
-        <v>0.5080450522928399</v>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>1D25215013008SXC11</t>
-        </is>
-      </c>
-      <c r="B120" t="n">
-        <v>26000</v>
-      </c>
-      <c r="C120" t="n">
-        <v>0.4863904532046125</v>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>1D25215Z13008QXPC0</t>
-        </is>
-      </c>
-      <c r="B121" t="n">
-        <v>5148</v>
-      </c>
-      <c r="C121" t="n">
         <v>0.5044194153928667</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated cbc.py file as per config params- days, input demand file, etc
</commit_message>
<xml_diff>
--- a/load_demand.xlsx
+++ b/load_demand.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C98"/>
+  <dimension ref="A1:C155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -440,10 +440,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>532</v>
+        <v>3000</v>
       </c>
       <c r="C2" t="n">
-        <v>0.5045669080182354</v>
+        <v>0.02380196511055731</v>
       </c>
     </row>
     <row r="3">
@@ -453,10 +453,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1512</v>
+        <v>9000</v>
       </c>
       <c r="C3" t="n">
-        <v>0.5151997854652722</v>
+        <v>0.07142176859950158</v>
       </c>
     </row>
     <row r="4">
@@ -466,10 +466,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>104</v>
+        <v>2218</v>
       </c>
       <c r="C4" t="n">
-        <v>0.5041324751944221</v>
+        <v>0.5052302417498691</v>
       </c>
     </row>
     <row r="5">
@@ -479,10 +479,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>873</v>
+        <v>2000</v>
       </c>
       <c r="C5" t="n">
-        <v>0.504792169482435</v>
+        <v>0.01586533119573327</v>
       </c>
     </row>
     <row r="6">
@@ -492,10 +492,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3577</v>
+        <v>5500</v>
       </c>
       <c r="C6" t="n">
-        <v>0.4306114239742558</v>
+        <v>0.5436435498976174</v>
       </c>
     </row>
     <row r="7">
@@ -505,1193 +505,1934 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>54776</v>
+        <v>67939</v>
       </c>
       <c r="C7" t="n">
-        <v>0.6340842048806651</v>
+        <v>0.5391910982714011</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1225219015008SLTB0</t>
+          <t>1225170016012LSTL0</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>70</v>
+        <v>654</v>
       </c>
       <c r="C8" t="n">
-        <v>0.3342611960311075</v>
+        <v>0.2551826219463801</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1225219015010QSTL0</t>
+          <t>1225175016014JSTL0</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>365</v>
+        <v>176</v>
       </c>
       <c r="C9" t="n">
-        <v>0.5077768838830786</v>
+        <v>0.2513889109350942</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1225220Z16008RXC10</t>
+          <t>1225216Z13008RXC10</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>36</v>
+        <v>100</v>
       </c>
       <c r="C10" t="n">
-        <v>0.3339823008849557</v>
+        <v>0.2507857267575676</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1225221615008QXC10</t>
+          <t>1225219015008SLTB0</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>375</v>
+        <v>915</v>
       </c>
       <c r="C11" t="n">
-        <v>0.3349825690533655</v>
+        <v>0.2572540833981492</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1225221715115SSTL0</t>
+          <t>1225219015010QSTL0</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3408</v>
+        <v>3000</v>
       </c>
       <c r="C12" t="n">
-        <v>0.5205604719764012</v>
+        <v>0.02380196511055731</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1225221716010SXC10</t>
+          <t>1225220Z16008RXC10</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>68</v>
+        <v>756</v>
       </c>
       <c r="C13" t="n">
-        <v>0.5</v>
+        <v>0.2559921586056921</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1225222716121NXC11</t>
+          <t>1225221615008QXC10</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>1191</v>
       </c>
       <c r="C14" t="n">
-        <v>0.4172030034861893</v>
+        <v>0.2594445943586406</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1225223516121PSKP0</t>
+          <t>1225221715115SSTL0</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>11420</v>
+        <v>9000</v>
       </c>
       <c r="C15" t="n">
-        <v>0.5080986859747921</v>
+        <v>0.07142176859950158</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1325114812074TUHL0</t>
+          <t>1225221716010SXC10</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>14986</v>
+        <v>990</v>
       </c>
       <c r="C16" t="n">
-        <v>0.553633681952266</v>
+        <v>0.507849330941761</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1325119015008SRBT0</t>
+          <t>1225222615008RXC10</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3263</v>
+        <v>650</v>
       </c>
       <c r="C17" t="n">
-        <v>0.5321802091713597</v>
+        <v>0.2551508754107208</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1325119815106QBRQ0</t>
+          <t>1225222716121MXC11</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>561</v>
+        <v>1149</v>
       </c>
       <c r="C18" t="n">
-        <v>0.5001582193617592</v>
+        <v>0.009111255734218004</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1325121715100SBRT0</t>
+          <t>1225222716121NXC11</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1519</v>
+        <v>520</v>
       </c>
       <c r="C19" t="n">
-        <v>0.5107267363904532</v>
+        <v>0.5034841822886078</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1325121715100SRBT0</t>
+          <t>1225223516121PSKP0</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1228</v>
+        <v>4555</v>
       </c>
       <c r="C20" t="n">
-        <v>0.5122526146419952</v>
+        <v>0.5032064001015889</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1325121715100SRXT0</t>
+          <t>1225223516121RBVN0</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>700</v>
+        <v>1544</v>
       </c>
       <c r="C21" t="n">
-        <v>0.5085492089031912</v>
+        <v>0.2622462261305735</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1325121715115SLTB0</t>
+          <t>1325114612069TUHL0</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1342</v>
+        <v>1400</v>
       </c>
       <c r="C22" t="n">
-        <v>0.5127916331456155</v>
+        <v>0.01110335084683884</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1325123715105SBRT0</t>
+          <t>1325114613071TTMX0</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1252</v>
+        <v>22</v>
       </c>
       <c r="C23" t="n">
-        <v>0.5174309466344864</v>
+        <v>0.0001666693122113049</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1325123715105SRXT0</t>
+          <t>1325114812074TUHL0</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>150</v>
+        <v>19500</v>
       </c>
       <c r="C24" t="n">
-        <v>0.502413515687852</v>
+        <v>0.1547564247051541</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1325213612065SULX1</t>
+          <t>1325119015008SRBT0</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>752</v>
+        <v>12000</v>
       </c>
       <c r="C25" t="n">
-        <v>0.5020166264414052</v>
+        <v>0.09523167034397371</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1325213615099MSXT0</t>
+          <t>1325119815106QBRQ0</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>4249</v>
+        <v>12650</v>
       </c>
       <c r="C26" t="n">
-        <v>0.4394609814963797</v>
+        <v>0.6003904823886094</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1325214613071TTMX0</t>
+          <t>1325121715100SBRT0</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>89</v>
+        <v>4000</v>
       </c>
       <c r="C27" t="n">
-        <v>0.5007750067042103</v>
+        <v>0.03173859902538136</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1325214812074TUHL0</t>
+          <t>1325121715100SRBT0</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>24182</v>
+        <v>4535</v>
       </c>
       <c r="C28" t="n">
-        <v>0.5724054706355591</v>
+        <v>0.03598469816981222</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1325214813075STMX0</t>
+          <t>1325121715100SRXT0</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1506</v>
+        <v>3188</v>
       </c>
       <c r="C29" t="n">
-        <v>0.5077768838830786</v>
+        <v>0.02529405228654423</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1325214813075SUNE1</t>
+          <t>1325121715115SLTB0</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>66042</v>
+        <v>4790</v>
       </c>
       <c r="C30" t="n">
-        <v>0.6166666666666667</v>
+        <v>0.03800853981809235</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1325215513073TUHL0</t>
+          <t>1325123715105SBRT0</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>39</v>
+        <v>6500</v>
       </c>
       <c r="C31" t="n">
-        <v>0.5207750067042103</v>
+        <v>0.05158018381244147</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1325215613075TTMX0</t>
+          <t>1325123715105SRXT0</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1418</v>
+        <v>513</v>
       </c>
       <c r="C32" t="n">
-        <v>0.5113676588897828</v>
+        <v>0.004063556564389911</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1325215613075TUHL0</t>
+          <t>1325213612065SULX1</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>3888</v>
+        <v>1263</v>
       </c>
       <c r="C33" t="n">
-        <v>0.5246714936980423</v>
+        <v>0.5087223606723916</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1325215813079STMX0</t>
+          <t>1325213615099MSXT0</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>4671</v>
+        <v>8250</v>
       </c>
       <c r="C34" t="n">
-        <v>0.526816840976133</v>
+        <v>0.5654692931633836</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1325215813079SUHL0</t>
+          <t>1325214612069TUHL0</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>7101</v>
+        <v>424</v>
       </c>
       <c r="C35" t="n">
-        <v>0.5321802091713597</v>
+        <v>0.003357196145970571</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>1325216513077TUHL0</t>
+          <t>1325214613071TTMX0</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1679</v>
+        <v>430</v>
       </c>
       <c r="C36" t="n">
-        <v>0.5080584607133279</v>
+        <v>0.003404815949459516</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1325216514079TTMX0</t>
+          <t>1325214812074TTMX0</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>5305</v>
+        <v>5000</v>
       </c>
       <c r="C37" t="n">
-        <v>0.5142611960311075</v>
+        <v>0.0396752329402054</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>1325216614081STMX0</t>
+          <t>1325214813075STMX0</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>6451</v>
+        <v>3890</v>
       </c>
       <c r="C38" t="n">
-        <v>0.5177902923035667</v>
+        <v>0.03086556929475071</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>1325216614081SUTR0</t>
+          <t>1325214813075SUNE1</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>5866</v>
+        <v>60594</v>
       </c>
       <c r="C39" t="n">
-        <v>0.5157307589165996</v>
+        <v>0.9801584152129399</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>1325216614081TVECE</t>
+          <t>1325215513073TUHL0</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>290</v>
+        <v>7340</v>
       </c>
       <c r="C40" t="n">
-        <v>0.3341110217216412</v>
+        <v>0.05824695630089366</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>1325216813083TUNE0</t>
+          <t>1325215513077HUNE0</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>2344</v>
+        <v>6</v>
       </c>
       <c r="C41" t="n">
-        <v>0.5107267363904532</v>
+        <v>0.2500396831695741</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>1325216814085STMX0</t>
+          <t>1325215613075TTMX0</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>14000</v>
+        <v>4122</v>
       </c>
       <c r="C42" t="n">
-        <v>0.5375435773665862</v>
+        <v>0.03270686836298989</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>1325216814085SURL0</t>
+          <t>1325215613075TUHL0</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>427</v>
+        <v>5000</v>
       </c>
       <c r="C43" t="n">
-        <v>0.5162939125770984</v>
+        <v>0.0396752329402054</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>1325216814085SUTR0</t>
+          <t>1325215813079STMX0</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>4582</v>
+        <v>10030</v>
       </c>
       <c r="C44" t="n">
-        <v>0.5138938053097345</v>
+        <v>0.2502301623835299</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>1325216814085TURL0</t>
+          <t>1325215813079SUHL0</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>5113</v>
+        <v>12000</v>
       </c>
       <c r="C45" t="n">
-        <v>0.5137114507910968</v>
+        <v>0.09523167034397371</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>1325216814085TURS0</t>
+          <t>1325216513077TUHL0</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>300</v>
+        <v>2950</v>
       </c>
       <c r="C46" t="n">
-        <v>0.500804505229284</v>
+        <v>0.253563548627756</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>1325217413077TUSP0</t>
+          <t>1325216514079TTMX0</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>3263</v>
+        <v>1044</v>
       </c>
       <c r="C47" t="n">
-        <v>0.5152936444086886</v>
+        <v>0.2507857267575676</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>1325217415081HUTR0</t>
+          <t>1325216614081STMX0</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1524</v>
+        <v>10094</v>
       </c>
       <c r="C48" t="n">
-        <v>0.5040868865647626</v>
+        <v>0.08010444610231908</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>1325217514082HURL2</t>
+          <t>1325216614081SUTR0</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>1868</v>
+        <v>15000</v>
       </c>
       <c r="C49" t="n">
-        <v>0.3396674711718959</v>
+        <v>0.1190415720884459</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>1325217514082TTMX0</t>
+          <t>1325216614081TVECE</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>6492</v>
+        <v>4194</v>
       </c>
       <c r="C50" t="n">
-        <v>0.5174094931617056</v>
+        <v>0.2832783060048572</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>1325217514082TUTR0</t>
+          <t>1325216813083TUNE0</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>2515</v>
+        <v>4050</v>
       </c>
       <c r="C51" t="n">
-        <v>0.5067444355054974</v>
+        <v>0.2503888950618264</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>1325217514082TVECH</t>
+          <t>1325216814085STMX0</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>2124</v>
+        <v>13500</v>
       </c>
       <c r="C52" t="n">
-        <v>0.5</v>
+        <v>0.1071366212162098</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>1325217613082TUNE0</t>
+          <t>1325216814085SURL0</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>2824</v>
+        <v>16000</v>
       </c>
       <c r="C53" t="n">
-        <v>0.3446017699115044</v>
+        <v>0.1269782060032699</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>1325217613082TUNE2</t>
+          <t>1325216814085SUTR0</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>2618</v>
+        <v>10000</v>
       </c>
       <c r="C54" t="n">
-        <v>0.3403539823008849</v>
+        <v>0.07935840251432563</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>1325217614084HURL2</t>
+          <t>1325216814085TURL0</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>895</v>
+        <v>7650</v>
       </c>
       <c r="C55" t="n">
-        <v>0.3368061142397425</v>
+        <v>0.06070731281448912</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>1325218415084TTMX0</t>
+          <t>1325216814085TURP0</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>90</v>
+        <v>1000</v>
       </c>
       <c r="C56" t="n">
-        <v>0.5041753821399839</v>
+        <v>0.007928697280909223</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>1325218416086VURL0</t>
+          <t>1325217413077TUSP0</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>2500</v>
+        <v>6106</v>
       </c>
       <c r="C57" t="n">
-        <v>0.4233708769106999</v>
+        <v>0.0484531500500008</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>1325218514086HURL0</t>
+          <t>1325217415081HUTR0</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>2500</v>
+        <v>1724</v>
       </c>
       <c r="C58" t="n">
-        <v>0.5067042102440332</v>
+        <v>0.01367482023524183</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>1325218515088HTMX0</t>
+          <t>1325217514082HURL1</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>11421</v>
+        <v>216</v>
       </c>
       <c r="C59" t="n">
-        <v>0.5321802091713597</v>
+        <v>0.2517063762916872</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>1325218515088HURP0</t>
+          <t>1325217514082HURL2</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>456</v>
+        <v>7888</v>
       </c>
       <c r="C60" t="n">
-        <v>0.5012228479485117</v>
+        <v>0.3125962316862173</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>1325218515088HUTR0</t>
+          <t>1325217514082HURP0</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>4924</v>
+        <v>340</v>
       </c>
       <c r="C61" t="n">
-        <v>0.5132046124966478</v>
+        <v>0.002690518897125351</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>1325218515088TURL0</t>
+          <t>1325217514082HVECL</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>2136</v>
+        <v>10201</v>
       </c>
       <c r="C62" t="n">
-        <v>0.505728077232502</v>
+        <v>0.3309536659312052</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>1325218614088HURL0</t>
+          <t>1325217514082TTMX0</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>676</v>
+        <v>5300</v>
       </c>
       <c r="C63" t="n">
-        <v>0.5027728613569321</v>
+        <v>0.2523730535405324</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>1325218615089HURL0</t>
+          <t>1325217514082TUTR0</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>1314</v>
+        <v>3824</v>
       </c>
       <c r="C64" t="n">
-        <v>0.5035237329042639</v>
+        <v>0.03034175145637232</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>1325219316087VURP0</t>
+          <t>1325217514082TVECH</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>609</v>
+        <v>1761</v>
       </c>
       <c r="C65" t="n">
-        <v>0.5016331456154465</v>
+        <v>0.5139605390561754</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>1325219316087VUTR0</t>
+          <t>1325217514086VURL0</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>6044</v>
+        <v>1323</v>
       </c>
       <c r="C66" t="n">
-        <v>0.5187717886832931</v>
+        <v>0.2604922300353974</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>1325219415088VURL1</t>
+          <t>1325217515084HURL4</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>2000</v>
+        <v>378</v>
       </c>
       <c r="C67" t="n">
-        <v>0.5053633681952266</v>
+        <v>0.2529921109858886</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>1325219416089HRHE0</t>
+          <t>1325217613082TUNE0</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>15404</v>
+        <v>10603</v>
       </c>
       <c r="C68" t="n">
-        <v>0.5134084204880665</v>
+        <v>0.3341441927649645</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>1325219515091VZEP0</t>
+          <t>1325217613082TUNE2</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>951</v>
+        <v>11900</v>
       </c>
       <c r="C69" t="n">
-        <v>0.3358836149101636</v>
+        <v>0.3444380069524913</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>1325220316091VURL1</t>
+          <t>1325217613082TUXPE</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>2761</v>
+        <v>3</v>
       </c>
       <c r="C70" t="n">
-        <v>0.505374094931617</v>
+        <v>0.2500158732678296</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>1325220416092VURL0</t>
+          <t>1325217614084HURL1</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>859</v>
+        <v>751</v>
       </c>
       <c r="C71" t="n">
-        <v>0.5</v>
+        <v>0.005952475436118034</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>1325220416092VURP0</t>
+          <t>1325217614084HURL2</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>536</v>
+        <v>22850</v>
       </c>
       <c r="C72" t="n">
-        <v>0.5014373826763208</v>
+        <v>0.4313441483198146</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>1325220515094VTMX0</t>
+          <t>1325218414082HUSP0</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>651</v>
+        <v>1386</v>
       </c>
       <c r="C73" t="n">
-        <v>0.5017457763475462</v>
+        <v>0.2609922379720313</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>1325220515094VUTR0</t>
+          <t>1325218414086VURL0</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>6098</v>
+        <v>909</v>
       </c>
       <c r="C74" t="n">
-        <v>0.5163529096272459</v>
+        <v>0.2572064635946603</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>1325220515094VZEP0</t>
+          <t>1325218415084TTMX0</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>558</v>
+        <v>650</v>
       </c>
       <c r="C75" t="n">
-        <v>0.5</v>
+        <v>0.253563548627756</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>1325220516095HTMX0</t>
+          <t>1325218415088VLHP0</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>4999</v>
+        <v>60</v>
       </c>
       <c r="C76" t="n">
-        <v>0.5134084204880665</v>
+        <v>0.2504682614009746</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>1325220516095HUTR0</t>
+          <t>1325218416086VURL0</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>742</v>
+        <v>2500</v>
       </c>
       <c r="C77" t="n">
-        <v>0.5042531509788147</v>
+        <v>0.01983364815314529</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>1325221317098VUX10</t>
+          <t>1325218514086HURL0</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>102</v>
+        <v>5312</v>
       </c>
       <c r="C78" t="n">
-        <v>0.5000107267363905</v>
+        <v>0.2723098779345704</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>1325221416095VURL0</t>
+          <t>1325218515088HTMX0</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>11230</v>
+        <v>11800</v>
       </c>
       <c r="C79" t="n">
-        <v>0.5321802091713597</v>
+        <v>0.2523730535405324</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>1325221417100HURL1</t>
+          <t>1325218515088HURL1</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>17000</v>
+        <v>2150</v>
       </c>
       <c r="C80" t="n">
-        <v>0.5455886296594261</v>
+        <v>0.2670558262829569</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>1325221417100HURS0</t>
+          <t>1325218515088HUTR0</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>143</v>
+        <v>253</v>
       </c>
       <c r="C81" t="n">
-        <v>0.500804505229284</v>
+        <v>0.002000031746535659</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>1325221715100SRHT0</t>
+          <t>1325218515088TURL0</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>19000</v>
+        <v>5000</v>
       </c>
       <c r="C82" t="n">
-        <v>0.5509519978546528</v>
+        <v>0.0396752329402054</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>1325221715100SRXT0</t>
+          <t>1325218515092VLHP0</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>308</v>
+        <v>60</v>
       </c>
       <c r="C83" t="n">
-        <v>0.5107267363904532</v>
+        <v>0.2504682614009746</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>1325222317101VUX10</t>
+          <t>1325218614088HURL0</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>456</v>
+        <v>3442</v>
       </c>
       <c r="C84" t="n">
-        <v>0.334556181281845</v>
+        <v>0.2535000555564374</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>1325222417099HURL0</t>
+          <t>1325218614088TVECE</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>2421</v>
+        <v>2840</v>
       </c>
       <c r="C85" t="n">
-        <v>0.5067042102440332</v>
+        <v>0.2725321036841855</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>1325223517104HRHT0</t>
+          <t>1325218614092VURL0</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>8000</v>
+        <v>275</v>
       </c>
       <c r="C86" t="n">
-        <v>0.5214534727809064</v>
+        <v>0.2521746376926618</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>1325223517104HRPG0</t>
+          <t>1325218615089HURL0</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>579</v>
+        <v>2000</v>
       </c>
       <c r="C87" t="n">
-        <v>0.5015526950925181</v>
+        <v>0.01586533119573327</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>1325223715105SRXT0</t>
+          <t>1325219316087VURL1</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>982</v>
+        <v>94</v>
       </c>
       <c r="C88" t="n">
-        <v>0.508779833735586</v>
+        <v>0.2507381069540786</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>1325226517112HRHT0</t>
+          <t>1325219316087VURP0</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>3325</v>
+        <v>94</v>
       </c>
       <c r="C89" t="n">
-        <v>0.5053633681952266</v>
+        <v>0.0007381069540786362</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>1425118916008QRBT0</t>
+          <t>1325219316087VUTR0</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>9000</v>
+        <v>7000</v>
       </c>
       <c r="C90" t="n">
-        <v>0.5241351568785197</v>
+        <v>0.05554850076985349</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>1D25115013008QXPC0</t>
+          <t>1325219415088VURL1</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>471</v>
+        <v>2000</v>
       </c>
       <c r="C91" t="n">
-        <v>0.50402252614642</v>
+        <v>0.01586533119573327</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>1D25212812074FXC10</t>
+          <t>1325219416089HRHE0</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>18658</v>
+        <v>14900</v>
       </c>
       <c r="C92" t="n">
-        <v>0.4980825958702065</v>
+        <v>0.5785647391228432</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>1D25212812086FXPC0</t>
+          <t>1325219416089VURL0</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>18100</v>
+        <v>372</v>
       </c>
       <c r="C93" t="n">
-        <v>0.4858541163850899</v>
+        <v>0.2529444911823997</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>1D25213812090FXPC0</t>
+          <t>1325219515091VURL0</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>19334</v>
+        <v>350</v>
       </c>
       <c r="C94" t="n">
-        <v>0.4945427728613569</v>
+        <v>0.2527698852362736</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>1D25214012006QXC10</t>
+          <t>1325219515091VZEP0</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>300</v>
+        <v>1421</v>
       </c>
       <c r="C95" t="n">
-        <v>0.5</v>
+        <v>0.2612700201590502</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>1D25214012008QSTL0</t>
+          <t>1325219515095VLHP0</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>2206</v>
+        <v>240</v>
       </c>
       <c r="C96" t="n">
-        <v>0.5080450522928399</v>
+        <v>0.2518968555056429</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>1D25215013008SXC11</t>
+          <t>1325219614095SU210</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>24086</v>
+        <v>339</v>
       </c>
       <c r="C97" t="n">
-        <v>0.4863904532046125</v>
+        <v>0.2526825822632106</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
+          <t>1325220316091VURL1</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>2214</v>
+      </c>
+      <c r="C98" t="n">
+        <v>0.2607858854902459</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>1325220316094VUX10</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>80</v>
+      </c>
+      <c r="C99" t="n">
+        <v>0.2506269940792711</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>1325220416092VURL0</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>587</v>
+      </c>
+      <c r="C100" t="n">
+        <v>0.2534841822886078</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>1325220416092VURP0</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>593</v>
+      </c>
+      <c r="C101" t="n">
+        <v>0.004698487277575835</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>1325220515094VTMX0</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>1396</v>
+      </c>
+      <c r="C102" t="n">
+        <v>0.25157939014905</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>1325220515094VURL1</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>100</v>
+      </c>
+      <c r="C103" t="n">
+        <v>0.2507857267575676</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>1325220515094VUTR0</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>4000</v>
+      </c>
+      <c r="C104" t="n">
+        <v>0.03173859902538136</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>1325220515094VZEP0</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>1330</v>
+      </c>
+      <c r="C105" t="n">
+        <v>0.2600636518039969</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>1325220516095HTMX0</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>5100</v>
+      </c>
+      <c r="C106" t="n">
+        <v>0.2507857267575676</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>1325220516095HUTR0</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>2578</v>
+      </c>
+      <c r="C107" t="n">
+        <v>0.2523730535405324</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>1325221117091YLEV0</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>29</v>
+      </c>
+      <c r="C108" t="n">
+        <v>0.2502222257496151</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>1325221217095YLEV0</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>52</v>
+      </c>
+      <c r="C109" t="n">
+        <v>0.250404768329656</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>1325221317094VURL2</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>60</v>
+      </c>
+      <c r="C110" t="n">
+        <v>0.2504682614009746</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>1325221317098VUX10</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>375</v>
+      </c>
+      <c r="C111" t="n">
+        <v>0.2529286179145701</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>1325221318095HURL0</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>104</v>
+      </c>
+      <c r="C112" t="n">
+        <v>0.2508174732932269</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>1325221318095HURL1</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>40</v>
+      </c>
+      <c r="C113" t="n">
+        <v>0.2503095287226781</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>1325221416095VURL0</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>12125</v>
+      </c>
+      <c r="C114" t="n">
+        <v>0.2515000238099017</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>1325221416095VURL2</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>425</v>
+      </c>
+      <c r="C115" t="n">
+        <v>0.2533651327798854</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>1325221416095VURS0</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>43</v>
+      </c>
+      <c r="C116" t="n">
+        <v>0.0003333386244226099</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>1325221416099WLHP0</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>12</v>
+      </c>
+      <c r="C117" t="n">
+        <v>0.2500873029730631</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>1325221417096HRHT0</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>32</v>
+      </c>
+      <c r="C118" t="n">
+        <v>0.2502460356513596</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>1325221417096HURL0</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>310</v>
+      </c>
+      <c r="C119" t="n">
+        <v>0.2524524198796806</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>1325221417096HURL3</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>498</v>
+      </c>
+      <c r="C120" t="n">
+        <v>0.2539445070556676</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>1325221417100HURL1</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>17000</v>
+      </c>
+      <c r="C121" t="n">
+        <v>0.1349148399180939</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>1325221417100HURS0</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>164</v>
+      </c>
+      <c r="C122" t="n">
+        <v>0.001293671328116319</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>1325221616100SRAB0</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>50</v>
+      </c>
+      <c r="C123" t="n">
+        <v>0.2503888950618264</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>1325221715100SRHT0</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>18500</v>
+      </c>
+      <c r="C124" t="n">
+        <v>0.14681979079033</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>1325221715100SRXT0</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>4000</v>
+      </c>
+      <c r="C125" t="n">
+        <v>0.03173859902538136</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>1325222118095YLEV1</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>50</v>
+      </c>
+      <c r="C126" t="n">
+        <v>0.2503888950618264</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>1325222217098VUX10</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>190</v>
+      </c>
+      <c r="C127" t="n">
+        <v>0.2515000238099017</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>1325222317101VUX10</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>622</v>
+      </c>
+      <c r="C128" t="n">
+        <v>0.2549286496611057</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>1325222417099HURL0</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>2882</v>
+      </c>
+      <c r="C129" t="n">
+        <v>0.2530238575215479</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>1325222517102SRAB0</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>100</v>
+      </c>
+      <c r="C130" t="n">
+        <v>0.2507857267575676</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>1325223118098VUX10</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>90</v>
+      </c>
+      <c r="C131" t="n">
+        <v>0.2507063604184193</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>1325223317103VUX11</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>584</v>
+      </c>
+      <c r="C132" t="n">
+        <v>0.2546270575723424</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>1325223418103HRHP0</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>2500</v>
+      </c>
+      <c r="C133" t="n">
+        <v>0.01983364815314529</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>1325223517104HBHT0</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>100</v>
+      </c>
+      <c r="C134" t="n">
+        <v>0.2507857267575676</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>1325223517104HRHT0</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>8380</v>
+      </c>
+      <c r="C135" t="n">
+        <v>0.2530079842537183</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>1325223517104HRHT3</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>12</v>
+      </c>
+      <c r="C136" t="n">
+        <v>0.2500873029730631</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>1325223517104HRPG0</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>602</v>
+      </c>
+      <c r="C137" t="n">
+        <v>0.004769916982809251</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>1325223616105HRHT0</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C138" t="n">
+        <v>0.0396752329402054</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>1325223715105SRXT0</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>3309</v>
+      </c>
+      <c r="C139" t="n">
+        <v>0.02625438499023794</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>1325223916120QRAB0</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
+        <v>1160</v>
+      </c>
+      <c r="C140" t="n">
+        <v>0.2591985587072811</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>1325224716111SELS0</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>50</v>
+      </c>
+      <c r="C141" t="n">
+        <v>0.2503888950618264</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>1325226517112HBHT0</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>75</v>
+      </c>
+      <c r="C142" t="n">
+        <v>0.250587310909697</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>1325226517112HRHT0</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>3669</v>
+      </c>
+      <c r="C143" t="n">
+        <v>0.2632383053699265</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>1325226517112HRPG0</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>108</v>
+      </c>
+      <c r="C144" t="n">
+        <v>0.2508492198288862</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>1325226517112TRAB0</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>21</v>
+      </c>
+      <c r="C145" t="n">
+        <v>0.2501587326782965</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>1325226616112TRAB0</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>50</v>
+      </c>
+      <c r="C146" t="n">
+        <v>0.2503888950618264</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>1425118916008QRBT0</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>9000</v>
+      </c>
+      <c r="C147" t="n">
+        <v>0.07142176859950158</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>1D25114012008QSTL0</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C148" t="n">
+        <v>0.02380196511055731</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>1D25115013008QXPC0</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>589</v>
+      </c>
+      <c r="C149" t="n">
+        <v>0.004666740741916539</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>1D25212812074FXC10</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>26070</v>
+      </c>
+      <c r="C150" t="n">
+        <v>0.706900109525548</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>1D25212812086FXPC0</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>18590</v>
+      </c>
+      <c r="C151" t="n">
+        <v>0.6475340878426642</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>1D25213812090FXPC0</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>33000</v>
+      </c>
+      <c r="C152" t="n">
+        <v>0.7619009825552787</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>1D25214012008QSTL0</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C153" t="n">
+        <v>0.02380196511055731</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>1D25215013008SXC11</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>33001</v>
+      </c>
+      <c r="C154" t="n">
+        <v>0.7619009825552787</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
           <t>1D25215Z13008QXPC0</t>
         </is>
       </c>
-      <c r="B98" t="n">
-        <v>2338</v>
-      </c>
-      <c r="C98" t="n">
-        <v>0.5044194153928667</v>
+      <c r="B155" t="n">
+        <v>6092</v>
+      </c>
+      <c r="C155" t="n">
+        <v>0.5303814346259464</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Everything done as per Version1- cbc
</commit_message>
<xml_diff>
--- a/load_demand.xlsx
+++ b/load_demand.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C155"/>
+  <dimension ref="A1:C97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -440,7 +440,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3000</v>
+        <v>1206</v>
       </c>
       <c r="C2" t="n">
         <v>0.02380196511055731</v>
@@ -453,7 +453,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>9000</v>
+        <v>3720</v>
       </c>
       <c r="C3" t="n">
         <v>0.07142176859950158</v>
@@ -466,7 +466,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2218</v>
+        <v>934</v>
       </c>
       <c r="C4" t="n">
         <v>0.5052302417498691</v>
@@ -479,7 +479,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2000</v>
+        <v>620</v>
       </c>
       <c r="C5" t="n">
         <v>0.01586533119573327</v>
@@ -492,7 +492,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5500</v>
+        <v>2135</v>
       </c>
       <c r="C6" t="n">
         <v>0.5436435498976174</v>
@@ -505,7 +505,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>67939</v>
+        <v>53874</v>
       </c>
       <c r="C7" t="n">
         <v>0.5391910982714011</v>
@@ -514,1924 +514,1170 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1225170016012LSTL0</t>
+          <t>1225216Z13008RXC10</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>654</v>
+        <v>100</v>
       </c>
       <c r="C8" t="n">
-        <v>0.2551826219463801</v>
+        <v>0.2507857267575676</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1225175016014JSTL0</t>
+          <t>1225219015010QSTL0</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>176</v>
+        <v>734</v>
       </c>
       <c r="C9" t="n">
-        <v>0.2513889109350942</v>
+        <v>0.02380196511055731</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1225216Z13008RXC10</t>
+          <t>1225220Z16008RXC10</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>100</v>
+        <v>324</v>
       </c>
       <c r="C10" t="n">
-        <v>0.2507857267575676</v>
+        <v>0.2559921586056921</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1225219015008SLTB0</t>
+          <t>1225221615008QXC10</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>915</v>
+        <v>36</v>
       </c>
       <c r="C11" t="n">
-        <v>0.2572540833981492</v>
+        <v>0.2594445943586406</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1225219015010QSTL0</t>
+          <t>1225221715115SSTL0</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3000</v>
+        <v>4661</v>
       </c>
       <c r="C12" t="n">
-        <v>0.02380196511055731</v>
+        <v>0.07142176859950158</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1225220Z16008RXC10</t>
+          <t>1225221716010SXC10</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>756</v>
+        <v>454</v>
       </c>
       <c r="C13" t="n">
-        <v>0.2559921586056921</v>
+        <v>0.507849330941761</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1225221615008QXC10</t>
+          <t>1225222615008RXC10</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1191</v>
+        <v>124</v>
       </c>
       <c r="C14" t="n">
-        <v>0.2594445943586406</v>
+        <v>0.2551508754107208</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1225221715115SSTL0</t>
+          <t>1225223516121PSKP0</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>9000</v>
+        <v>4555</v>
       </c>
       <c r="C15" t="n">
-        <v>0.07142176859950158</v>
+        <v>0.5032064001015889</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1225221716010SXC10</t>
+          <t>1325114812074TUHL0</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>990</v>
+        <v>19452</v>
       </c>
       <c r="C16" t="n">
-        <v>0.507849330941761</v>
+        <v>0.1547564247051541</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1225222615008RXC10</t>
+          <t>1325119015008SRBT0</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>650</v>
+        <v>2313</v>
       </c>
       <c r="C17" t="n">
-        <v>0.2551508754107208</v>
+        <v>0.09523167034397371</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1225222716121MXC11</t>
+          <t>1325119815106QBRQ0</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1149</v>
+        <v>3495</v>
       </c>
       <c r="C18" t="n">
-        <v>0.009111255734218004</v>
+        <v>0.6003904823886094</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1225222716121NXC11</t>
+          <t>1325121715100SBRT0</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>520</v>
+        <v>1130</v>
       </c>
       <c r="C19" t="n">
-        <v>0.5034841822886078</v>
+        <v>0.03173859902538136</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1225223516121PSKP0</t>
+          <t>1325121715100SRBT0</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>4555</v>
+        <v>2557</v>
       </c>
       <c r="C20" t="n">
-        <v>0.5032064001015889</v>
+        <v>0.03598469816981222</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1225223516121RBVN0</t>
+          <t>1325121715100SRXT0</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1544</v>
+        <v>574</v>
       </c>
       <c r="C21" t="n">
-        <v>0.2622462261305735</v>
+        <v>0.02529405228654423</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1325114612069TUHL0</t>
+          <t>1325121715115SLTB0</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1400</v>
+        <v>1129</v>
       </c>
       <c r="C22" t="n">
-        <v>0.01110335084683884</v>
+        <v>0.03800853981809235</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1325114613071TTMX0</t>
+          <t>1325123715105SBRT0</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>22</v>
+        <v>3595</v>
       </c>
       <c r="C23" t="n">
-        <v>0.0001666693122113049</v>
+        <v>0.05158018381244147</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1325114812074TUHL0</t>
+          <t>1325213612065SULX1</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>19500</v>
+        <v>888</v>
       </c>
       <c r="C24" t="n">
-        <v>0.1547564247051541</v>
+        <v>0.5087223606723916</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1325119015008SRBT0</t>
+          <t>1325213615099MSXT0</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>12000</v>
+        <v>5754</v>
       </c>
       <c r="C25" t="n">
-        <v>0.09523167034397371</v>
+        <v>0.5654692931633836</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1325119815106QBRQ0</t>
+          <t>1325214613071TTMX0</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>12650</v>
+        <v>213</v>
       </c>
       <c r="C26" t="n">
-        <v>0.6003904823886094</v>
+        <v>0.003404815949459516</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1325121715100SBRT0</t>
+          <t>1325214813075STMX0</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>4000</v>
+        <v>3890</v>
       </c>
       <c r="C27" t="n">
-        <v>0.03173859902538136</v>
+        <v>0.03086556929475071</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1325121715100SRBT0</t>
+          <t>1325214813075SUNE1</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>4535</v>
+        <v>60594</v>
       </c>
       <c r="C28" t="n">
-        <v>0.03598469816981222</v>
+        <v>0.9801584152129399</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1325121715100SRXT0</t>
+          <t>1325215613075TTMX0</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>3188</v>
+        <v>3603</v>
       </c>
       <c r="C29" t="n">
-        <v>0.02529405228654423</v>
+        <v>0.03270686836298989</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1325121715115SLTB0</t>
+          <t>1325215613075TUHL0</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>4790</v>
+        <v>4530</v>
       </c>
       <c r="C30" t="n">
-        <v>0.03800853981809235</v>
+        <v>0.0396752329402054</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1325123715105SBRT0</t>
+          <t>1325215813079STMX0</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>6500</v>
+        <v>9652</v>
       </c>
       <c r="C31" t="n">
-        <v>0.05158018381244147</v>
+        <v>0.2502301623835299</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1325123715105SRXT0</t>
+          <t>1325215813079SUHL0</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>513</v>
+        <v>11375</v>
       </c>
       <c r="C32" t="n">
-        <v>0.004063556564389911</v>
+        <v>0.09523167034397371</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1325213612065SULX1</t>
+          <t>1325216513077TUHL0</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1263</v>
+        <v>2451</v>
       </c>
       <c r="C33" t="n">
-        <v>0.5087223606723916</v>
+        <v>0.253563548627756</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1325213615099MSXT0</t>
+          <t>1325216514079TTMX0</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>8250</v>
+        <v>304</v>
       </c>
       <c r="C34" t="n">
-        <v>0.5654692931633836</v>
+        <v>0.2507857267575676</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1325214612069TUHL0</t>
+          <t>1325216614081STMX0</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>424</v>
+        <v>7810</v>
       </c>
       <c r="C35" t="n">
-        <v>0.003357196145970571</v>
+        <v>0.08010444610231908</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>1325214613071TTMX0</t>
+          <t>1325216614081SUTR0</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>430</v>
+        <v>7916</v>
       </c>
       <c r="C36" t="n">
-        <v>0.003404815949459516</v>
+        <v>0.1190415720884459</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1325214812074TTMX0</t>
+          <t>1325216614081TVECE</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>5000</v>
+        <v>2623</v>
       </c>
       <c r="C37" t="n">
-        <v>0.0396752329402054</v>
+        <v>0.2832783060048572</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>1325214813075STMX0</t>
+          <t>1325216813083TUNE0</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>3890</v>
+        <v>2541</v>
       </c>
       <c r="C38" t="n">
-        <v>0.03086556929475071</v>
+        <v>0.2503888950618264</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>1325214813075SUNE1</t>
+          <t>1325216814085STMX0</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>60594</v>
+        <v>11729</v>
       </c>
       <c r="C39" t="n">
-        <v>0.9801584152129399</v>
+        <v>0.1071366212162098</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>1325215513073TUHL0</t>
+          <t>1325216814085SUTR0</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>7340</v>
+        <v>3943</v>
       </c>
       <c r="C40" t="n">
-        <v>0.05824695630089366</v>
+        <v>0.07935840251432563</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>1325215513077HUNE0</t>
+          <t>1325216814085TURL0</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>6</v>
+        <v>5349</v>
       </c>
       <c r="C41" t="n">
-        <v>0.2500396831695741</v>
+        <v>0.06070731281448912</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>1325215613075TTMX0</t>
+          <t>1325217413077TUSP0</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>4122</v>
+        <v>5581</v>
       </c>
       <c r="C42" t="n">
-        <v>0.03270686836298989</v>
+        <v>0.0484531500500008</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>1325215613075TUHL0</t>
+          <t>1325217415081HUTR0</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>5000</v>
+        <v>1724</v>
       </c>
       <c r="C43" t="n">
-        <v>0.0396752329402054</v>
+        <v>0.01367482023524183</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>1325215813079STMX0</t>
+          <t>1325217514082HURL1</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>10030</v>
+        <v>215</v>
       </c>
       <c r="C44" t="n">
-        <v>0.2502301623835299</v>
+        <v>0.2517063762916872</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>1325215813079SUHL0</t>
+          <t>1325217514082HURL2</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>12000</v>
+        <v>6830</v>
       </c>
       <c r="C45" t="n">
-        <v>0.09523167034397371</v>
+        <v>0.3125962316862173</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>1325216513077TUHL0</t>
+          <t>1325217514082HVECL</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>2950</v>
+        <v>7695</v>
       </c>
       <c r="C46" t="n">
-        <v>0.253563548627756</v>
+        <v>0.3309536659312052</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>1325216514079TTMX0</t>
+          <t>1325217514082TTMX0</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>1044</v>
+        <v>4150</v>
       </c>
       <c r="C47" t="n">
-        <v>0.2507857267575676</v>
+        <v>0.2523730535405324</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>1325216614081STMX0</t>
+          <t>1325217514082TUTR0</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>10094</v>
+        <v>2696</v>
       </c>
       <c r="C48" t="n">
-        <v>0.08010444610231908</v>
+        <v>0.03034175145637232</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>1325216614081SUTR0</t>
+          <t>1325217514082TVECH</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>15000</v>
+        <v>505</v>
       </c>
       <c r="C49" t="n">
-        <v>0.1190415720884459</v>
+        <v>0.5139605390561754</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>1325216614081TVECE</t>
+          <t>1325217613082TUNE0</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>4194</v>
+        <v>10323</v>
       </c>
       <c r="C50" t="n">
-        <v>0.2832783060048572</v>
+        <v>0.3341441927649645</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>1325216813083TUNE0</t>
+          <t>1325217613082TUNE2</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>4050</v>
+        <v>11900</v>
       </c>
       <c r="C51" t="n">
-        <v>0.2503888950618264</v>
+        <v>0.3444380069524913</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>1325216814085STMX0</t>
+          <t>1325217614084HURL2</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>13500</v>
+        <v>22753</v>
       </c>
       <c r="C52" t="n">
-        <v>0.1071366212162098</v>
+        <v>0.4313441483198146</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>1325216814085SURL0</t>
+          <t>1325218416086VURL0</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>16000</v>
+        <v>1348</v>
       </c>
       <c r="C53" t="n">
-        <v>0.1269782060032699</v>
+        <v>0.01983364815314529</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>1325216814085SUTR0</t>
+          <t>1325218514086HURL0</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>10000</v>
+        <v>1680</v>
       </c>
       <c r="C54" t="n">
-        <v>0.07935840251432563</v>
+        <v>0.2723098779345704</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>1325216814085TURL0</t>
+          <t>1325218515088HTMX0</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>7650</v>
+        <v>11800</v>
       </c>
       <c r="C55" t="n">
-        <v>0.06070731281448912</v>
+        <v>0.2523730535405324</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>1325216814085TURP0</t>
+          <t>1325218515088HURL1</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>1000</v>
+        <v>2150</v>
       </c>
       <c r="C56" t="n">
-        <v>0.007928697280909223</v>
+        <v>0.2670558262829569</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>1325217413077TUSP0</t>
+          <t>1325218515088HUTR0</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>6106</v>
+        <v>253</v>
       </c>
       <c r="C57" t="n">
-        <v>0.0484531500500008</v>
+        <v>0.002000031746535659</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>1325217415081HUTR0</t>
+          <t>1325218515088TURL0</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>1724</v>
+        <v>5000</v>
       </c>
       <c r="C58" t="n">
-        <v>0.01367482023524183</v>
+        <v>0.0396752329402054</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>1325217514082HURL1</t>
+          <t>1325218614088HURL0</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>216</v>
+        <v>2035</v>
       </c>
       <c r="C59" t="n">
-        <v>0.2517063762916872</v>
+        <v>0.2535000555564374</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>1325217514082HURL2</t>
+          <t>1325218615089HURL0</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>7888</v>
+        <v>2000</v>
       </c>
       <c r="C60" t="n">
-        <v>0.3125962316862173</v>
+        <v>0.01586533119573327</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>1325217514082HURP0</t>
+          <t>1325219316087VURP0</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>340</v>
+        <v>33</v>
       </c>
       <c r="C61" t="n">
-        <v>0.002690518897125351</v>
+        <v>0.0007381069540786362</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>1325217514082HVECL</t>
+          <t>1325219316087VUTR0</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>10201</v>
+        <v>3599</v>
       </c>
       <c r="C62" t="n">
-        <v>0.3309536659312052</v>
+        <v>0.05554850076985349</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>1325217514082TTMX0</t>
+          <t>1325219415088VURL1</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>5300</v>
+        <v>2000</v>
       </c>
       <c r="C63" t="n">
-        <v>0.2523730535405324</v>
+        <v>0.01586533119573327</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>1325217514082TUTR0</t>
+          <t>1325219416089HRHE0</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>3824</v>
+        <v>11727</v>
       </c>
       <c r="C64" t="n">
-        <v>0.03034175145637232</v>
+        <v>0.5785647391228432</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>1325217514082TVECH</t>
+          <t>1325219515091VURL0</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>1761</v>
+        <v>338</v>
       </c>
       <c r="C65" t="n">
-        <v>0.5139605390561754</v>
+        <v>0.2527698852362736</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>1325217514086VURL0</t>
+          <t>1325219515091VZEP0</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>1323</v>
+        <v>1421</v>
       </c>
       <c r="C66" t="n">
-        <v>0.2604922300353974</v>
+        <v>0.2612700201590502</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>1325217515084HURL4</t>
+          <t>1325220316091VURL1</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>378</v>
+        <v>2214</v>
       </c>
       <c r="C67" t="n">
-        <v>0.2529921109858886</v>
+        <v>0.2607858854902459</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>1325217613082TUNE0</t>
+          <t>1325220316094VUX10</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>10603</v>
+        <v>78</v>
       </c>
       <c r="C68" t="n">
-        <v>0.3341441927649645</v>
+        <v>0.2506269940792711</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>1325217613082TUNE2</t>
+          <t>1325220416092VURL0</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>11900</v>
+        <v>587</v>
       </c>
       <c r="C69" t="n">
-        <v>0.3444380069524913</v>
+        <v>0.2534841822886078</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>1325217613082TUXPE</t>
+          <t>1325220416092VURP0</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>3</v>
+        <v>593</v>
       </c>
       <c r="C70" t="n">
-        <v>0.2500158732678296</v>
+        <v>0.004698487277575835</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>1325217614084HURL1</t>
+          <t>1325220515094VTMX0</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>751</v>
+        <v>1396</v>
       </c>
       <c r="C71" t="n">
-        <v>0.005952475436118034</v>
+        <v>0.25157939014905</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>1325217614084HURL2</t>
+          <t>1325220515094VURL1</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>22850</v>
+        <v>100</v>
       </c>
       <c r="C72" t="n">
-        <v>0.4313441483198146</v>
+        <v>0.2507857267575676</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>1325218414082HUSP0</t>
+          <t>1325220515094VUTR0</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>1386</v>
+        <v>4000</v>
       </c>
       <c r="C73" t="n">
-        <v>0.2609922379720313</v>
+        <v>0.03173859902538136</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>1325218414086VURL0</t>
+          <t>1325220515094VZEP0</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>909</v>
+        <v>1330</v>
       </c>
       <c r="C74" t="n">
-        <v>0.2572064635946603</v>
+        <v>0.2600636518039969</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>1325218415084TTMX0</t>
+          <t>1325220516095HTMX0</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>650</v>
+        <v>3869</v>
       </c>
       <c r="C75" t="n">
-        <v>0.253563548627756</v>
+        <v>0.2507857267575676</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>1325218415088VLHP0</t>
+          <t>1325220516095HUTR0</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>60</v>
+        <v>1153</v>
       </c>
       <c r="C76" t="n">
-        <v>0.2504682614009746</v>
+        <v>0.2523730535405324</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>1325218416086VURL0</t>
+          <t>1325221317098VUX10</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>2500</v>
+        <v>375</v>
       </c>
       <c r="C77" t="n">
-        <v>0.01983364815314529</v>
+        <v>0.2529286179145701</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>1325218514086HURL0</t>
+          <t>1325221416095VURL0</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>5312</v>
+        <v>10401</v>
       </c>
       <c r="C78" t="n">
-        <v>0.2723098779345704</v>
+        <v>0.2515000238099017</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>1325218515088HTMX0</t>
+          <t>1325221417096HRHT0</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>11800</v>
+        <v>32</v>
       </c>
       <c r="C79" t="n">
-        <v>0.2523730535405324</v>
+        <v>0.2502460356513596</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>1325218515088HURL1</t>
+          <t>1325221417100HURL1</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>2150</v>
+        <v>17000</v>
       </c>
       <c r="C80" t="n">
-        <v>0.2670558262829569</v>
+        <v>0.1349148399180939</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>1325218515088HUTR0</t>
+          <t>1325221417100HURS0</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>253</v>
+        <v>164</v>
       </c>
       <c r="C81" t="n">
-        <v>0.002000031746535659</v>
+        <v>0.001293671328116319</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>1325218515088TURL0</t>
+          <t>1325221715100SRHT0</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>5000</v>
+        <v>18500</v>
       </c>
       <c r="C82" t="n">
-        <v>0.0396752329402054</v>
+        <v>0.14681979079033</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>1325218515092VLHP0</t>
+          <t>1325221715100SRXT0</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>60</v>
+        <v>1118</v>
       </c>
       <c r="C83" t="n">
-        <v>0.2504682614009746</v>
+        <v>0.03173859902538136</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>1325218614088HURL0</t>
+          <t>1325222317101VUX10</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>3442</v>
+        <v>622</v>
       </c>
       <c r="C84" t="n">
-        <v>0.2535000555564374</v>
+        <v>0.2549286496611057</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>1325218614088TVECE</t>
+          <t>1325222417099HURL0</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>2840</v>
+        <v>2882</v>
       </c>
       <c r="C85" t="n">
-        <v>0.2725321036841855</v>
+        <v>0.2530238575215479</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>1325218614092VURL0</t>
+          <t>1325223517104HRHT0</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>275</v>
+        <v>8380</v>
       </c>
       <c r="C86" t="n">
-        <v>0.2521746376926618</v>
+        <v>0.2530079842537183</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>1325218615089HURL0</t>
+          <t>1325223517104HRPG0</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>2000</v>
+        <v>602</v>
       </c>
       <c r="C87" t="n">
-        <v>0.01586533119573327</v>
+        <v>0.004769916982809251</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>1325219316087VURL1</t>
+          <t>1325223715105SRXT0</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>94</v>
+        <v>300</v>
       </c>
       <c r="C88" t="n">
-        <v>0.2507381069540786</v>
+        <v>0.02625438499023794</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>1325219316087VURP0</t>
+          <t>1325226517112HRHT0</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>94</v>
+        <v>3669</v>
       </c>
       <c r="C89" t="n">
-        <v>0.0007381069540786362</v>
+        <v>0.2632383053699265</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>1325219316087VUTR0</t>
+          <t>1425118916008QRBT0</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>7000</v>
+        <v>8850</v>
       </c>
       <c r="C90" t="n">
-        <v>0.05554850076985349</v>
+        <v>0.07142176859950158</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>1325219415088VURL1</t>
+          <t>1D25115013008QXPC0</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>2000</v>
+        <v>339</v>
       </c>
       <c r="C91" t="n">
-        <v>0.01586533119573327</v>
+        <v>0.004666740741916539</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>1325219416089HRHE0</t>
+          <t>1D25212812074FXC10</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>14900</v>
+        <v>18150</v>
       </c>
       <c r="C92" t="n">
-        <v>0.5785647391228432</v>
+        <v>0.706900109525548</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>1325219416089VURL0</t>
+          <t>1D25212812086FXPC0</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>372</v>
+        <v>11650</v>
       </c>
       <c r="C93" t="n">
-        <v>0.2529444911823997</v>
+        <v>0.6475340878426642</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>1325219515091VURL0</t>
+          <t>1D25213812090FXPC0</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>350</v>
+        <v>26561</v>
       </c>
       <c r="C94" t="n">
-        <v>0.2527698852362736</v>
+        <v>0.7619009825552787</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>1325219515091VZEP0</t>
+          <t>1D25214012008QSTL0</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>1421</v>
+        <v>1724</v>
       </c>
       <c r="C95" t="n">
-        <v>0.2612700201590502</v>
+        <v>0.02380196511055731</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>1325219515095VLHP0</t>
+          <t>1D25215013008SXC11</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>240</v>
+        <v>22290</v>
       </c>
       <c r="C96" t="n">
-        <v>0.2518968555056429</v>
+        <v>0.7619009825552787</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>1325219614095SU210</t>
+          <t>1D25215Z13008QXPC0</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>339</v>
+        <v>3226</v>
       </c>
       <c r="C97" t="n">
-        <v>0.2526825822632106</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>1325220316091VURL1</t>
-        </is>
-      </c>
-      <c r="B98" t="n">
-        <v>2214</v>
-      </c>
-      <c r="C98" t="n">
-        <v>0.2607858854902459</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>1325220316094VUX10</t>
-        </is>
-      </c>
-      <c r="B99" t="n">
-        <v>80</v>
-      </c>
-      <c r="C99" t="n">
-        <v>0.2506269940792711</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>1325220416092VURL0</t>
-        </is>
-      </c>
-      <c r="B100" t="n">
-        <v>587</v>
-      </c>
-      <c r="C100" t="n">
-        <v>0.2534841822886078</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>1325220416092VURP0</t>
-        </is>
-      </c>
-      <c r="B101" t="n">
-        <v>593</v>
-      </c>
-      <c r="C101" t="n">
-        <v>0.004698487277575835</v>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>1325220515094VTMX0</t>
-        </is>
-      </c>
-      <c r="B102" t="n">
-        <v>1396</v>
-      </c>
-      <c r="C102" t="n">
-        <v>0.25157939014905</v>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>1325220515094VURL1</t>
-        </is>
-      </c>
-      <c r="B103" t="n">
-        <v>100</v>
-      </c>
-      <c r="C103" t="n">
-        <v>0.2507857267575676</v>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>1325220515094VUTR0</t>
-        </is>
-      </c>
-      <c r="B104" t="n">
-        <v>4000</v>
-      </c>
-      <c r="C104" t="n">
-        <v>0.03173859902538136</v>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>1325220515094VZEP0</t>
-        </is>
-      </c>
-      <c r="B105" t="n">
-        <v>1330</v>
-      </c>
-      <c r="C105" t="n">
-        <v>0.2600636518039969</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>1325220516095HTMX0</t>
-        </is>
-      </c>
-      <c r="B106" t="n">
-        <v>5100</v>
-      </c>
-      <c r="C106" t="n">
-        <v>0.2507857267575676</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>1325220516095HUTR0</t>
-        </is>
-      </c>
-      <c r="B107" t="n">
-        <v>2578</v>
-      </c>
-      <c r="C107" t="n">
-        <v>0.2523730535405324</v>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>1325221117091YLEV0</t>
-        </is>
-      </c>
-      <c r="B108" t="n">
-        <v>29</v>
-      </c>
-      <c r="C108" t="n">
-        <v>0.2502222257496151</v>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>1325221217095YLEV0</t>
-        </is>
-      </c>
-      <c r="B109" t="n">
-        <v>52</v>
-      </c>
-      <c r="C109" t="n">
-        <v>0.250404768329656</v>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>1325221317094VURL2</t>
-        </is>
-      </c>
-      <c r="B110" t="n">
-        <v>60</v>
-      </c>
-      <c r="C110" t="n">
-        <v>0.2504682614009746</v>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>1325221317098VUX10</t>
-        </is>
-      </c>
-      <c r="B111" t="n">
-        <v>375</v>
-      </c>
-      <c r="C111" t="n">
-        <v>0.2529286179145701</v>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>1325221318095HURL0</t>
-        </is>
-      </c>
-      <c r="B112" t="n">
-        <v>104</v>
-      </c>
-      <c r="C112" t="n">
-        <v>0.2508174732932269</v>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>1325221318095HURL1</t>
-        </is>
-      </c>
-      <c r="B113" t="n">
-        <v>40</v>
-      </c>
-      <c r="C113" t="n">
-        <v>0.2503095287226781</v>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>1325221416095VURL0</t>
-        </is>
-      </c>
-      <c r="B114" t="n">
-        <v>12125</v>
-      </c>
-      <c r="C114" t="n">
-        <v>0.2515000238099017</v>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>1325221416095VURL2</t>
-        </is>
-      </c>
-      <c r="B115" t="n">
-        <v>425</v>
-      </c>
-      <c r="C115" t="n">
-        <v>0.2533651327798854</v>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>1325221416095VURS0</t>
-        </is>
-      </c>
-      <c r="B116" t="n">
-        <v>43</v>
-      </c>
-      <c r="C116" t="n">
-        <v>0.0003333386244226099</v>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>1325221416099WLHP0</t>
-        </is>
-      </c>
-      <c r="B117" t="n">
-        <v>12</v>
-      </c>
-      <c r="C117" t="n">
-        <v>0.2500873029730631</v>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>1325221417096HRHT0</t>
-        </is>
-      </c>
-      <c r="B118" t="n">
-        <v>32</v>
-      </c>
-      <c r="C118" t="n">
-        <v>0.2502460356513596</v>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>1325221417096HURL0</t>
-        </is>
-      </c>
-      <c r="B119" t="n">
-        <v>310</v>
-      </c>
-      <c r="C119" t="n">
-        <v>0.2524524198796806</v>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>1325221417096HURL3</t>
-        </is>
-      </c>
-      <c r="B120" t="n">
-        <v>498</v>
-      </c>
-      <c r="C120" t="n">
-        <v>0.2539445070556676</v>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>1325221417100HURL1</t>
-        </is>
-      </c>
-      <c r="B121" t="n">
-        <v>17000</v>
-      </c>
-      <c r="C121" t="n">
-        <v>0.1349148399180939</v>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>1325221417100HURS0</t>
-        </is>
-      </c>
-      <c r="B122" t="n">
-        <v>164</v>
-      </c>
-      <c r="C122" t="n">
-        <v>0.001293671328116319</v>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>1325221616100SRAB0</t>
-        </is>
-      </c>
-      <c r="B123" t="n">
-        <v>50</v>
-      </c>
-      <c r="C123" t="n">
-        <v>0.2503888950618264</v>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>1325221715100SRHT0</t>
-        </is>
-      </c>
-      <c r="B124" t="n">
-        <v>18500</v>
-      </c>
-      <c r="C124" t="n">
-        <v>0.14681979079033</v>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>1325221715100SRXT0</t>
-        </is>
-      </c>
-      <c r="B125" t="n">
-        <v>4000</v>
-      </c>
-      <c r="C125" t="n">
-        <v>0.03173859902538136</v>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>1325222118095YLEV1</t>
-        </is>
-      </c>
-      <c r="B126" t="n">
-        <v>50</v>
-      </c>
-      <c r="C126" t="n">
-        <v>0.2503888950618264</v>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>1325222217098VUX10</t>
-        </is>
-      </c>
-      <c r="B127" t="n">
-        <v>190</v>
-      </c>
-      <c r="C127" t="n">
-        <v>0.2515000238099017</v>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>1325222317101VUX10</t>
-        </is>
-      </c>
-      <c r="B128" t="n">
-        <v>622</v>
-      </c>
-      <c r="C128" t="n">
-        <v>0.2549286496611057</v>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>1325222417099HURL0</t>
-        </is>
-      </c>
-      <c r="B129" t="n">
-        <v>2882</v>
-      </c>
-      <c r="C129" t="n">
-        <v>0.2530238575215479</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>1325222517102SRAB0</t>
-        </is>
-      </c>
-      <c r="B130" t="n">
-        <v>100</v>
-      </c>
-      <c r="C130" t="n">
-        <v>0.2507857267575676</v>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>1325223118098VUX10</t>
-        </is>
-      </c>
-      <c r="B131" t="n">
-        <v>90</v>
-      </c>
-      <c r="C131" t="n">
-        <v>0.2507063604184193</v>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>1325223317103VUX11</t>
-        </is>
-      </c>
-      <c r="B132" t="n">
-        <v>584</v>
-      </c>
-      <c r="C132" t="n">
-        <v>0.2546270575723424</v>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="inlineStr">
-        <is>
-          <t>1325223418103HRHP0</t>
-        </is>
-      </c>
-      <c r="B133" t="n">
-        <v>2500</v>
-      </c>
-      <c r="C133" t="n">
-        <v>0.01983364815314529</v>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t>1325223517104HBHT0</t>
-        </is>
-      </c>
-      <c r="B134" t="n">
-        <v>100</v>
-      </c>
-      <c r="C134" t="n">
-        <v>0.2507857267575676</v>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="inlineStr">
-        <is>
-          <t>1325223517104HRHT0</t>
-        </is>
-      </c>
-      <c r="B135" t="n">
-        <v>8380</v>
-      </c>
-      <c r="C135" t="n">
-        <v>0.2530079842537183</v>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t>1325223517104HRHT3</t>
-        </is>
-      </c>
-      <c r="B136" t="n">
-        <v>12</v>
-      </c>
-      <c r="C136" t="n">
-        <v>0.2500873029730631</v>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t>1325223517104HRPG0</t>
-        </is>
-      </c>
-      <c r="B137" t="n">
-        <v>602</v>
-      </c>
-      <c r="C137" t="n">
-        <v>0.004769916982809251</v>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="inlineStr">
-        <is>
-          <t>1325223616105HRHT0</t>
-        </is>
-      </c>
-      <c r="B138" t="n">
-        <v>5000</v>
-      </c>
-      <c r="C138" t="n">
-        <v>0.0396752329402054</v>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t>1325223715105SRXT0</t>
-        </is>
-      </c>
-      <c r="B139" t="n">
-        <v>3309</v>
-      </c>
-      <c r="C139" t="n">
-        <v>0.02625438499023794</v>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>1325223916120QRAB0</t>
-        </is>
-      </c>
-      <c r="B140" t="n">
-        <v>1160</v>
-      </c>
-      <c r="C140" t="n">
-        <v>0.2591985587072811</v>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>1325224716111SELS0</t>
-        </is>
-      </c>
-      <c r="B141" t="n">
-        <v>50</v>
-      </c>
-      <c r="C141" t="n">
-        <v>0.2503888950618264</v>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>1325226517112HBHT0</t>
-        </is>
-      </c>
-      <c r="B142" t="n">
-        <v>75</v>
-      </c>
-      <c r="C142" t="n">
-        <v>0.250587310909697</v>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>1325226517112HRHT0</t>
-        </is>
-      </c>
-      <c r="B143" t="n">
-        <v>3669</v>
-      </c>
-      <c r="C143" t="n">
-        <v>0.2632383053699265</v>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>1325226517112HRPG0</t>
-        </is>
-      </c>
-      <c r="B144" t="n">
-        <v>108</v>
-      </c>
-      <c r="C144" t="n">
-        <v>0.2508492198288862</v>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t>1325226517112TRAB0</t>
-        </is>
-      </c>
-      <c r="B145" t="n">
-        <v>21</v>
-      </c>
-      <c r="C145" t="n">
-        <v>0.2501587326782965</v>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>1325226616112TRAB0</t>
-        </is>
-      </c>
-      <c r="B146" t="n">
-        <v>50</v>
-      </c>
-      <c r="C146" t="n">
-        <v>0.2503888950618264</v>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>1425118916008QRBT0</t>
-        </is>
-      </c>
-      <c r="B147" t="n">
-        <v>9000</v>
-      </c>
-      <c r="C147" t="n">
-        <v>0.07142176859950158</v>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>1D25114012008QSTL0</t>
-        </is>
-      </c>
-      <c r="B148" t="n">
-        <v>3000</v>
-      </c>
-      <c r="C148" t="n">
-        <v>0.02380196511055731</v>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>1D25115013008QXPC0</t>
-        </is>
-      </c>
-      <c r="B149" t="n">
-        <v>589</v>
-      </c>
-      <c r="C149" t="n">
-        <v>0.004666740741916539</v>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>1D25212812074FXC10</t>
-        </is>
-      </c>
-      <c r="B150" t="n">
-        <v>26070</v>
-      </c>
-      <c r="C150" t="n">
-        <v>0.706900109525548</v>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>1D25212812086FXPC0</t>
-        </is>
-      </c>
-      <c r="B151" t="n">
-        <v>18590</v>
-      </c>
-      <c r="C151" t="n">
-        <v>0.6475340878426642</v>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>1D25213812090FXPC0</t>
-        </is>
-      </c>
-      <c r="B152" t="n">
-        <v>33000</v>
-      </c>
-      <c r="C152" t="n">
-        <v>0.7619009825552787</v>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>1D25214012008QSTL0</t>
-        </is>
-      </c>
-      <c r="B153" t="n">
-        <v>3000</v>
-      </c>
-      <c r="C153" t="n">
-        <v>0.02380196511055731</v>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>1D25215013008SXC11</t>
-        </is>
-      </c>
-      <c r="B154" t="n">
-        <v>33001</v>
-      </c>
-      <c r="C154" t="n">
-        <v>0.7619009825552787</v>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>1D25215Z13008QXPC0</t>
-        </is>
-      </c>
-      <c r="B155" t="n">
-        <v>6092</v>
-      </c>
-      <c r="C155" t="n">
         <v>0.5303814346259464</v>
       </c>
     </row>

</xml_diff>